<commit_message>
Padroniza o Kendall do T2 e ajusta o acabamento da planilha
A fila de capacidade ilimitada passa a aparecer como G/G/2/∞ em todos
os lugares (scripts, planilha e comentários dos .yml), igual ao desenho
da rede. Na planilha: índice do estado centralizado, rótulo da
conferência sem corte e perdas de uma simulação sem casas decimais. Os
valores não mudam (410 fórmulas, sem erros, 60 células da comparação
conferidas contra o analise_indices.py).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/T2 - Avaliação de Aprendizagem/indices_desempenho.xlsx
+++ b/T2 - Avaliação de Aprendizagem/indices_desempenho.xlsx
@@ -135,7 +135,7 @@
     <t xml:space="preserve">N1 - Triagem</t>
   </si>
   <si>
-    <t xml:space="preserve">G/G/2</t>
+    <t xml:space="preserve">G/G/2/∞</t>
   </si>
   <si>
     <t xml:space="preserve">∞</t>
@@ -264,14 +264,14 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="\+0.0%;\-0.0%;0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
-    <numFmt numFmtId="170" formatCode="0.0000"/>
-    <numFmt numFmtId="171" formatCode="#,##0.0000"/>
-    <numFmt numFmtId="172" formatCode="#,##0"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="0.0000"/>
+    <numFmt numFmtId="172" formatCode="#,##0.0000"/>
     <numFmt numFmtId="173" formatCode="0.00%"/>
   </numFmts>
   <fonts count="9">
@@ -386,7 +386,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -423,7 +423,83 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -431,83 +507,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -830,11 +838,11 @@
         <f aca="false">IF(C5=0,"-",D5/C5-1)</f>
         <v>-</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="6" t="n">
         <f aca="false">Sementes!$D$10</f>
         <v>0</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="6" t="n">
         <f aca="false">Sementes!$D$34</f>
         <v>0</v>
       </c>
@@ -850,11 +858,11 @@
       <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <f aca="false">Atual_Q1!$D$16</f>
         <v>1.41568125204773</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <f aca="false">Melhorado_Q1!$D$16</f>
         <v>1.39488508907472</v>
       </c>
@@ -862,11 +870,11 @@
         <f aca="false">IF(C6=0,"-",D6/C6-1)</f>
         <v>-0.0146898625258508</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <f aca="false">Sementes!$E$10</f>
         <v>1.41133983495493</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <f aca="false">Sementes!$E$34</f>
         <v>1.40072494018522</v>
       </c>
@@ -882,11 +890,11 @@
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <f aca="false">Atual_Q1!$E$16</f>
         <v>10.41706305183</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="7" t="n">
         <f aca="false">Melhorado_Q1!$E$16</f>
         <v>10.3139826700539</v>
       </c>
@@ -894,11 +902,11 @@
         <f aca="false">IF(C7=0,"-",D7/C7-1)</f>
         <v>-0.00989534010337156</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <f aca="false">Sementes!$F$10</f>
         <v>10.3932156484888</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="7" t="n">
         <f aca="false">Sementes!$F$34</f>
         <v>10.3374236778124</v>
       </c>
@@ -914,11 +922,11 @@
       <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <f aca="false">Atual_Q1!$F$16</f>
         <v>0.694470870122</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <f aca="false">Melhorado_Q1!$F$16</f>
         <v>0.687598844670259</v>
       </c>
@@ -926,11 +934,11 @@
         <f aca="false">IF(C8=0,"-",D8/C8-1)</f>
         <v>-0.00989534010337156</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <f aca="false">Sementes!$G$10</f>
         <v>0.692881043232584</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <f aca="false">Sementes!$G$34</f>
         <v>0.689161578520829</v>
       </c>
@@ -946,11 +954,11 @@
       <c r="B9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="9" t="n">
         <f aca="false">Atual_Q1!$B$19</f>
         <v>8.15401372730886</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">Melhorado_Q1!$B$19</f>
         <v>8.11452840496641</v>
       </c>
@@ -958,11 +966,11 @@
         <f aca="false">IF(C9=0,"-",D9/C9-1)</f>
         <v>-0.00484244001334144</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <f aca="false">Sementes!$H$10</f>
         <v>8.14765033515906</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <f aca="false">Sementes!$H$34</f>
         <v>8.12999321936416</v>
       </c>
@@ -990,11 +998,11 @@
         <f aca="false">IF(C11=0,"-",D11/C11-1)</f>
         <v>-0.99076324744774</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="6" t="n">
         <f aca="false">Sementes!$D$18</f>
         <v>2249.4</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="6" t="n">
         <f aca="false">Sementes!$D$42</f>
         <v>30</v>
       </c>
@@ -1010,11 +1018,11 @@
       <c r="B12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="7" t="n">
         <f aca="false">Atual_Q2!$D$22</f>
         <v>8.17396989080396</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="7" t="n">
         <f aca="false">Melhorado_Q2!$D$22</f>
         <v>2.60866603726796</v>
       </c>
@@ -1022,11 +1030,11 @@
         <f aca="false">IF(C12=0,"-",D12/C12-1)</f>
         <v>-0.68085690648276</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="7" t="n">
         <f aca="false">Sementes!$E$18</f>
         <v>8.33877105333836</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <f aca="false">Sementes!$E$42</f>
         <v>2.84210013133221</v>
       </c>
@@ -1042,11 +1050,11 @@
       <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <f aca="false">Atual_Q2!$E$22</f>
         <v>3.99164297815367</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="7" t="n">
         <f aca="false">Melhorado_Q2!$E$22</f>
         <v>3.19126005156441</v>
       </c>
@@ -1054,11 +1062,11 @@
         <f aca="false">IF(C13=0,"-",D13/C13-1)</f>
         <v>-0.20051465799165</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="7" t="n">
         <f aca="false">Sementes!$F$18</f>
         <v>3.99480118198915</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="7" t="n">
         <f aca="false">Sementes!$F$42</f>
         <v>3.28272438294814</v>
       </c>
@@ -1074,11 +1082,11 @@
       <c r="B14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="8" t="n">
         <f aca="false">Atual_Q2!$F$22</f>
         <v>0.997910744538417</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <f aca="false">Melhorado_Q2!$F$22</f>
         <v>0.797815012891104</v>
       </c>
@@ -1086,11 +1094,11 @@
         <f aca="false">IF(C14=0,"-",D14/C14-1)</f>
         <v>-0.20051465799165</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="8" t="n">
         <f aca="false">Sementes!$G$18</f>
         <v>0.998700295497287</v>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="G14" s="8" t="n">
         <f aca="false">Sementes!$G$42</f>
         <v>0.820681095737036</v>
       </c>
@@ -1106,11 +1114,11 @@
       <c r="B15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="9" t="n">
         <f aca="false">Atual_Q2!$B$25</f>
         <v>122.866247340359</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="9" t="n">
         <f aca="false">Melhorado_Q2!$B$25</f>
         <v>49.0464455127524</v>
       </c>
@@ -1118,11 +1126,11 @@
         <f aca="false">IF(C15=0,"-",D15/C15-1)</f>
         <v>-0.60081432798313</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="9" t="n">
         <f aca="false">Sementes!$H$18</f>
         <v>125.243160894702</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="9" t="n">
         <f aca="false">Sementes!$H$42</f>
         <v>51.9187481907654</v>
       </c>
@@ -1150,11 +1158,11 @@
         <f aca="false">IF(C17=0,"-",D17/C17-1)</f>
         <v>-0.810126582278481</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" s="6" t="n">
         <f aca="false">Sementes!$D$26</f>
         <v>124.6</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" s="6" t="n">
         <f aca="false">Sementes!$D$50</f>
         <v>28.6</v>
       </c>
@@ -1170,11 +1178,11 @@
       <c r="B18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="7" t="n">
         <f aca="false">Atual_Q3!$D$17</f>
         <v>1.92326099427398</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="7" t="n">
         <f aca="false">Melhorado_Q3!$D$17</f>
         <v>1.30476270994767</v>
       </c>
@@ -1182,11 +1190,11 @@
         <f aca="false">IF(C18=0,"-",D18/C18-1)</f>
         <v>-0.321588326372621</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F18" s="7" t="n">
         <f aca="false">Sementes!$E$26</f>
         <v>2.13208122294476</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="7" t="n">
         <f aca="false">Sementes!$E$50</f>
         <v>1.38868662667366</v>
       </c>
@@ -1202,11 +1210,11 @@
       <c r="B19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="7" t="n">
         <f aca="false">Atual_Q3!$E$17</f>
         <v>1.11835315374716</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="7" t="n">
         <f aca="false">Melhorado_Q3!$E$17</f>
         <v>0.957204790250873</v>
       </c>
@@ -1214,11 +1222,11 @@
         <f aca="false">IF(C19=0,"-",D19/C19-1)</f>
         <v>-0.144094343505305</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F19" s="7" t="n">
         <f aca="false">Sementes!$F$26</f>
         <v>1.1533427305336</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="7" t="n">
         <f aca="false">Sementes!$F$50</f>
         <v>0.974159755102891</v>
       </c>
@@ -1234,11 +1242,11 @@
       <c r="B20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="8" t="n">
         <f aca="false">Atual_Q3!$F$17</f>
         <v>0.838764865310368</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="8" t="n">
         <f aca="false">Melhorado_Q3!$F$17</f>
         <v>0.717903592688155</v>
       </c>
@@ -1246,11 +1254,11 @@
         <f aca="false">IF(C20=0,"-",D20/C20-1)</f>
         <v>-0.144094343505305</v>
       </c>
-      <c r="F20" s="7" t="n">
+      <c r="F20" s="8" t="n">
         <f aca="false">Sementes!$G$26</f>
         <v>0.865007047900202</v>
       </c>
-      <c r="G20" s="7" t="n">
+      <c r="G20" s="8" t="n">
         <f aca="false">Sementes!$G$50</f>
         <v>0.730619816327168</v>
       </c>
@@ -1266,11 +1274,11 @@
       <c r="B21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="9" t="n">
         <f aca="false">Atual_Q3!$B$20</f>
         <v>103.183559924514</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="9" t="n">
         <f aca="false">Melhorado_Q3!$B$20</f>
         <v>81.7858031992739</v>
       </c>
@@ -1278,11 +1286,11 @@
         <f aca="false">IF(C21=0,"-",D21/C21-1)</f>
         <v>-0.207375639500072</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="9" t="n">
         <f aca="false">Sementes!$H$26</f>
         <v>110.85857041069</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="9" t="n">
         <f aca="false">Sementes!$H$50</f>
         <v>85.5027448181177</v>
       </c>
@@ -1391,33 +1399,33 @@
       <c r="D5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I5" s="12" t="n">
         <f aca="false">(G5+H5)/2</f>
         <v>8</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="13" t="n">
         <f aca="false">60/I5</f>
         <v>7.5</v>
       </c>
-      <c r="K5" s="10" t="n">
+      <c r="K5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="10" t="n">
+      <c r="L5" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="M5" s="10" t="n">
+      <c r="M5" s="11" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1434,23 +1442,23 @@
       <c r="D6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="I6" s="11" t="n">
+      <c r="I6" s="12" t="n">
         <f aca="false">(G6+H6)/2</f>
         <v>30</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="13" t="n">
         <f aca="false">60/I6</f>
         <v>2</v>
       </c>
@@ -1468,23 +1476,23 @@
       <c r="D7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="I7" s="12" t="n">
         <f aca="false">(G7+H7)/2</f>
         <v>45</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="13" t="n">
         <f aca="false">60/I7</f>
         <v>1.33333333333333</v>
       </c>
@@ -1502,33 +1510,33 @@
       <c r="D9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="I9" s="11" t="n">
+      <c r="I9" s="12" t="n">
         <f aca="false">(G9+H9)/2</f>
         <v>8</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="13" t="n">
         <f aca="false">60/I9</f>
         <v>7.5</v>
       </c>
-      <c r="K9" s="10" t="n">
+      <c r="K9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="L9" s="10" t="n">
+      <c r="L9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="M9" s="10" t="n">
+      <c r="M9" s="11" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1545,23 +1553,23 @@
       <c r="D10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="12" t="n">
         <f aca="false">(G10+H10)/2</f>
         <v>30</v>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="13" t="n">
         <f aca="false">60/I10</f>
         <v>2</v>
       </c>
@@ -1579,29 +1587,29 @@
       <c r="D11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G11" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="I11" s="11" t="n">
+      <c r="I11" s="12" t="n">
         <f aca="false">(G11+H11)/2</f>
         <v>45</v>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="13" t="n">
         <f aca="false">60/I11</f>
         <v>1.33333333333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1626,10 +1634,10 @@
       <c r="B16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="15" t="n">
         <v>0.45</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="15" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1640,11 +1648,11 @@
       <c r="B17" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="12" t="n">
         <f aca="false">1-SUM(C16)</f>
         <v>0.55</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="12" t="n">
         <f aca="false">1-SUM(D16)</f>
         <v>0.7</v>
       </c>
@@ -1656,10 +1664,10 @@
       <c r="B18" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="C18" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="16" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1670,10 +1678,10 @@
       <c r="B19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="16" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -1684,11 +1692,11 @@
       <c r="B20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C20" s="12" t="n">
         <f aca="false">1-SUM(C18:C19)</f>
         <v>0.6</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="12" t="n">
         <f aca="false">1-SUM(D18:D19)</f>
         <v>0.6</v>
       </c>
@@ -1700,10 +1708,10 @@
       <c r="B21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="C21" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="D21" s="16" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1714,11 +1722,11 @@
       <c r="B22" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C22" s="12" t="n">
         <f aca="false">1-SUM(C21)</f>
         <v>0.8</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D22" s="12" t="n">
         <f aca="false">1-SUM(D21)</f>
         <v>0.8</v>
       </c>
@@ -1747,7 +1755,7 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
@@ -1771,7 +1779,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <f aca="false">Parâmetros!$E$5</f>
         <v>2</v>
       </c>
@@ -1780,7 +1788,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16" t="str">
+      <c r="B5" s="17" t="str">
         <f aca="false">Parâmetros!$F$5</f>
         <v>∞</v>
       </c>
@@ -1789,7 +1797,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">Parâmetros!$J$5</f>
         <v>7.5</v>
       </c>
@@ -1798,7 +1806,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>146269.717459168</v>
       </c>
     </row>
@@ -1806,7 +1814,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1831,146 +1839,146 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>1799.95110185165</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.0123056989041776</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>85779.4168018978</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.586446861947644</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">C12*A12</f>
         <v>0.586446861947644</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>4.39835146460733</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.293223430973822</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>54849.1453557126</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.374986335575742</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">C13*A13</f>
         <v>0.749972671151484</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>5.62479503363613</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.374986335575742</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>3771.2275628848</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.025782695341143</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">C14*A14</f>
         <v>0.077348086023429</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.386740430117145</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.025782695341143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>69.9766368214041</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.00047840823129325</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">C15*A15</f>
         <v>0.001913632925173</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.00717612346939875</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.00047840823129325</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="23" t="n">
         <f aca="false">SUM(B11:B15)</f>
         <v>146269.717459168</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">SUM(C11:C15)</f>
         <v>1</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="25" t="n">
         <f aca="false">SUM(D11:D15)</f>
         <v>1.41568125204773</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="25" t="n">
         <f aca="false">SUM(E11:E15)</f>
         <v>10.41706305183</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F16" s="26" t="n">
         <f aca="false">SUM(F11:F15)</f>
         <v>0.694470870122</v>
       </c>
@@ -1979,16 +1987,16 @@
       <c r="A18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <f aca="false">D16/E16</f>
         <v>0.135900228788481</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="27" t="n">
         <f aca="false">B18*60</f>
         <v>8.15401372730886</v>
       </c>
@@ -2021,7 +2029,7 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
@@ -2045,7 +2053,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <f aca="false">Parâmetros!$E$6</f>
         <v>2</v>
       </c>
@@ -2054,7 +2062,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">Parâmetros!$F$6</f>
         <v>10</v>
       </c>
@@ -2063,7 +2071,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">Parâmetros!$J$6</f>
         <v>2</v>
       </c>
@@ -2072,7 +2080,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>146269.717459168</v>
       </c>
     </row>
@@ -2080,7 +2088,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>2057</v>
       </c>
     </row>
@@ -2105,290 +2113,290 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>68.9358042832464</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.000471292386973333</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>473.318003565073</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.00323592614921952</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">C12*A12</f>
         <v>0.00323592614921952</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.00647185229843903</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.00161796307460976</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>998.020987044089</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.00682315522570617</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">C13*A13</f>
         <v>0.0136463104514123</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.0272926209028247</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.00682315522570617</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>1917.09665392619</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.0131065861562312</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">C14*A14</f>
         <v>0.0393197584686936</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.0524263446249248</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.0131065861562312</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>3102.75989075005</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.0212125923577872</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">C15*A15</f>
         <v>0.0848503694311489</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.0848503694311489</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.0212125923577872</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="19" t="n">
         <v>5724.31662190985</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0391353502375351</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="13" t="n">
         <f aca="false">C16*A16</f>
         <v>0.195676751187675</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.15654140095014</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0391353502375351</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="19" t="n">
         <v>9481.77895309404</v>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="22" t="n">
         <f aca="false">B17/$B$7</f>
         <v>0.064823937024018</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="13" t="n">
         <f aca="false">C17*A17</f>
         <v>0.388943622144108</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="13" t="n">
         <f aca="false">C17*MIN(A17,$B$4)*$B$6</f>
         <v>0.259295748096072</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="13" t="n">
         <f aca="false">C17*MIN(A17,$B$4)/$B$4</f>
         <v>0.064823937024018</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="19" t="n">
         <v>16807.0212294292</v>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="22" t="n">
         <f aca="false">B18/$B$7</f>
         <v>0.114904311851979</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="13" t="n">
         <f aca="false">C18*A18</f>
         <v>0.804330182963855</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="13" t="n">
         <f aca="false">C18*MIN(A18,$B$4)*$B$6</f>
         <v>0.459617247407917</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="13" t="n">
         <f aca="false">C18*MIN(A18,$B$4)/$B$4</f>
         <v>0.114904311851979</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="19" t="n">
         <v>30899.1502329391</v>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="22" t="n">
         <f aca="false">B19/$B$7</f>
         <v>0.211247760436569</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <f aca="false">C19*A19</f>
         <v>1.68998208349255</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <f aca="false">C19*MIN(A19,$B$4)*$B$6</f>
         <v>0.844991041746277</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="13" t="n">
         <f aca="false">C19*MIN(A19,$B$4)/$B$4</f>
         <v>0.211247760436569</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="19" t="n">
         <v>43355.2211746937</v>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="22" t="n">
         <f aca="false">B20/$B$7</f>
         <v>0.296405995224517</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <f aca="false">C20*A20</f>
         <v>2.66765395702065</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="13" t="n">
         <f aca="false">C20*MIN(A20,$B$4)*$B$6</f>
         <v>1.18562398089807</v>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="13" t="n">
         <f aca="false">C20*MIN(A20,$B$4)/$B$4</f>
         <v>0.296405995224517</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="19" t="n">
         <v>33442.0979075339</v>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="22" t="n">
         <f aca="false">B21/$B$7</f>
         <v>0.228633092949464</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="13" t="n">
         <f aca="false">C21*A21</f>
         <v>2.28633092949464</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="13" t="n">
         <f aca="false">C21*MIN(A21,$B$4)*$B$6</f>
         <v>0.914532371797856</v>
       </c>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="13" t="n">
         <f aca="false">C21*MIN(A21,$B$4)/$B$4</f>
         <v>0.228633092949464</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="21" t="n">
+      <c r="B22" s="23" t="n">
         <f aca="false">SUM(B11:B21)</f>
         <v>146269.717459168</v>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="24" t="n">
         <f aca="false">SUM(C11:C21)</f>
         <v>1</v>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">SUM(D11:D21)</f>
         <v>8.17396989080396</v>
       </c>
-      <c r="E22" s="23" t="n">
+      <c r="E22" s="25" t="n">
         <f aca="false">SUM(E11:E21)</f>
         <v>3.99164297815367</v>
       </c>
-      <c r="F22" s="24" t="n">
+      <c r="F22" s="26" t="n">
         <f aca="false">SUM(F11:F21)</f>
         <v>0.997910744538417</v>
       </c>
@@ -2397,16 +2405,16 @@
       <c r="A24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="13" t="n">
         <f aca="false">D22/E22</f>
         <v>2.04777078900599</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="25" t="n">
+      <c r="B25" s="27" t="n">
         <f aca="false">B24*60</f>
         <v>122.866247340359</v>
       </c>
@@ -2439,7 +2447,7 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
@@ -2463,7 +2471,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <f aca="false">Parâmetros!$E$7</f>
         <v>1</v>
       </c>
@@ -2472,7 +2480,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">Parâmetros!$F$7</f>
         <v>5</v>
       </c>
@@ -2481,7 +2489,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">Parâmetros!$J$7</f>
         <v>1.33333333333333</v>
       </c>
@@ -2490,7 +2498,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>146269.717459168</v>
       </c>
     </row>
@@ -2498,7 +2506,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>79</v>
       </c>
     </row>
@@ -2523,170 +2531,170 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>23583.8175955433</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.161235134689631</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>41758.0095335674</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.285486362173525</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">C12*A12</f>
         <v>0.285486362173525</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.380648482898034</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.285486362173525</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>33814.2295845244</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.231177240046039</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">C13*A13</f>
         <v>0.462354480092077</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.308236320061385</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.231177240046039</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>23065.2667063912</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.15768996554485</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">C14*A14</f>
         <v>0.473069896634551</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.210253287393134</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.15768996554485</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>17509.3967848048</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.119706232355939</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">C15*A15</f>
         <v>0.478824929423756</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.159608309807919</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.119706232355939</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="19" t="n">
         <v>6538.99725433718</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0447050651900149</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="13" t="n">
         <f aca="false">C16*A16</f>
         <v>0.223525325950075</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.0596067535866866</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0447050651900149</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="23" t="n">
         <f aca="false">SUM(B11:B16)</f>
         <v>146269.717459168</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="24" t="n">
         <f aca="false">SUM(C11:C16)</f>
         <v>1</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="25" t="n">
         <f aca="false">SUM(D11:D16)</f>
         <v>1.92326099427398</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="25" t="n">
         <f aca="false">SUM(E11:E16)</f>
         <v>1.11835315374716</v>
       </c>
-      <c r="F17" s="24" t="n">
+      <c r="F17" s="26" t="n">
         <f aca="false">SUM(F11:F16)</f>
         <v>0.838764865310368</v>
       </c>
@@ -2695,16 +2703,16 @@
       <c r="A19" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <f aca="false">D17/E17</f>
         <v>1.7197259987419</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="27" t="n">
         <f aca="false">B19*60</f>
         <v>103.183559924514</v>
       </c>
@@ -2737,7 +2745,7 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
@@ -2761,7 +2769,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <f aca="false">Parâmetros!$E$9</f>
         <v>2</v>
       </c>
@@ -2770,7 +2778,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16" t="str">
+      <c r="B5" s="17" t="str">
         <f aca="false">Parâmetros!$F$9</f>
         <v>∞</v>
       </c>
@@ -2779,7 +2787,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">Parâmetros!$J$9</f>
         <v>7.5</v>
       </c>
@@ -2788,7 +2796,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>154191.662644958</v>
       </c>
     </row>
@@ -2796,7 +2804,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2821,146 +2829,146 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>1939.06857775338</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.0125757031508136</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>92461.1699494906</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.599650904357856</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">C12*A12</f>
         <v>0.599650904357856</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>4.49738178268392</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.299825452178928</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>56785.0519056795</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.368275761034063</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">C13*A13</f>
         <v>0.736551522068127</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>5.52413641551095</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.368275761034063</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>2977.11152589601</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.0193078631803271</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">C14*A14</f>
         <v>0.0579235895409813</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.289617947704907</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.0193078631803271</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>29.2606861386448</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.000189768276939983</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">C15*A15</f>
         <v>0.000759073107759931</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.00284652415409974</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.000189768276939983</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="23" t="n">
         <f aca="false">SUM(B11:B15)</f>
         <v>154191.662644958</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">SUM(C11:C15)</f>
         <v>1</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="25" t="n">
         <f aca="false">SUM(D11:D15)</f>
         <v>1.39488508907472</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="25" t="n">
         <f aca="false">SUM(E11:E15)</f>
         <v>10.3139826700539</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F16" s="26" t="n">
         <f aca="false">SUM(F11:F15)</f>
         <v>0.687598844670259</v>
       </c>
@@ -2969,16 +2977,16 @@
       <c r="A18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <f aca="false">D16/E16</f>
         <v>0.135242140082773</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="27" t="n">
         <f aca="false">B18*60</f>
         <v>8.11452840496641</v>
       </c>
@@ -3011,7 +3019,7 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
@@ -3035,7 +3043,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <f aca="false">Parâmetros!$E$10</f>
         <v>2</v>
       </c>
@@ -3044,7 +3052,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">Parâmetros!$F$10</f>
         <v>10</v>
       </c>
@@ -3053,7 +3061,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">Parâmetros!$J$10</f>
         <v>2</v>
       </c>
@@ -3062,7 +3070,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>154191.662644958</v>
       </c>
     </row>
@@ -3070,7 +3078,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3095,290 +3103,290 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>13755.7628458915</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.0892121053105547</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>34838.9529565573</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.225945763596683</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">C12*A12</f>
         <v>0.225945763596683</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.451891527193367</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.112972881798342</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>37189.4851482725</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.241189987255699</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">C13*A13</f>
         <v>0.482379974511398</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.964759949022796</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.241189987255699</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>28872.3286273032</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.187249609557585</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">C14*A14</f>
         <v>0.561748828672754</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.748998438230339</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.187249609557585</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>17039.0442472659</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.110505613306084</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">C15*A15</f>
         <v>0.442022453224336</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.442022453224336</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.110505613306084</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="19" t="n">
         <v>9475.65576402098</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0614537491942067</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="13" t="n">
         <f aca="false">C16*A16</f>
         <v>0.307268745971033</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.245814996776827</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0614537491942067</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="19" t="n">
         <v>5719.80337375123</v>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="22" t="n">
         <f aca="false">B17/$B$7</f>
         <v>0.0370954127845528</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="13" t="n">
         <f aca="false">C17*A17</f>
         <v>0.222572476707317</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="13" t="n">
         <f aca="false">C17*MIN(A17,$B$4)*$B$6</f>
         <v>0.148381651138211</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="13" t="n">
         <f aca="false">C17*MIN(A17,$B$4)/$B$4</f>
         <v>0.0370954127845528</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="19" t="n">
         <v>3614.86460275762</v>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="22" t="n">
         <f aca="false">B18/$B$7</f>
         <v>0.0234439692830942</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="13" t="n">
         <f aca="false">C18*A18</f>
         <v>0.164107784981659</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="13" t="n">
         <f aca="false">C18*MIN(A18,$B$4)*$B$6</f>
         <v>0.0937758771323767</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="13" t="n">
         <f aca="false">C18*MIN(A18,$B$4)/$B$4</f>
         <v>0.0234439692830942</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="19" t="n">
         <v>2269.19500326645</v>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="22" t="n">
         <f aca="false">B19/$B$7</f>
         <v>0.014716716613216</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <f aca="false">C19*A19</f>
         <v>0.117733732905728</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <f aca="false">C19*MIN(A19,$B$4)*$B$6</f>
         <v>0.0588668664528639</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="13" t="n">
         <f aca="false">C19*MIN(A19,$B$4)/$B$4</f>
         <v>0.014716716613216</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="19" t="n">
         <v>1076.94461905677</v>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="22" t="n">
         <f aca="false">B20/$B$7</f>
         <v>0.00698445428619927</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <f aca="false">C20*A20</f>
         <v>0.0628600885757934</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="13" t="n">
         <f aca="false">C20*MIN(A20,$B$4)*$B$6</f>
         <v>0.0279378171447971</v>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="13" t="n">
         <f aca="false">C20*MIN(A20,$B$4)/$B$4</f>
         <v>0.00698445428619927</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="19" t="n">
         <v>339.625456814654</v>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="22" t="n">
         <f aca="false">B21/$B$7</f>
         <v>0.00220261881212525</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="13" t="n">
         <f aca="false">C21*A21</f>
         <v>0.0220261881212525</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="13" t="n">
         <f aca="false">C21*MIN(A21,$B$4)*$B$6</f>
         <v>0.00881047524850098</v>
       </c>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="13" t="n">
         <f aca="false">C21*MIN(A21,$B$4)/$B$4</f>
         <v>0.00220261881212525</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="21" t="n">
+      <c r="B22" s="23" t="n">
         <f aca="false">SUM(B11:B21)</f>
         <v>154191.662644958</v>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="24" t="n">
         <f aca="false">SUM(C11:C21)</f>
         <v>1</v>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">SUM(D11:D21)</f>
         <v>2.60866603726796</v>
       </c>
-      <c r="E22" s="23" t="n">
+      <c r="E22" s="25" t="n">
         <f aca="false">SUM(E11:E21)</f>
         <v>3.19126005156441</v>
       </c>
-      <c r="F22" s="24" t="n">
+      <c r="F22" s="26" t="n">
         <f aca="false">SUM(F11:F21)</f>
         <v>0.797815012891104</v>
       </c>
@@ -3387,16 +3395,16 @@
       <c r="A24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="13" t="n">
         <f aca="false">D22/E22</f>
         <v>0.817440758545873</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="25" t="n">
+      <c r="B25" s="27" t="n">
         <f aca="false">B24*60</f>
         <v>49.0464455127524</v>
       </c>
@@ -3429,7 +3437,7 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
@@ -3453,7 +3461,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <f aca="false">Parâmetros!$E$11</f>
         <v>1</v>
       </c>
@@ -3462,7 +3470,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">Parâmetros!$F$11</f>
         <v>5</v>
       </c>
@@ -3471,7 +3479,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <f aca="false">Parâmetros!$J$11</f>
         <v>1.33333333333333</v>
       </c>
@@ -3480,7 +3488,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>154191.662644958</v>
       </c>
     </row>
@@ -3488,7 +3496,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3513,170 +3521,170 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>43496.9140695827</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.282096407311845</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="13" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>53992.8889684649</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.350167369897223</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <f aca="false">C12*A12</f>
         <v>0.350167369897223</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.466889826529631</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.350167369897223</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>33062.39108421</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.214423987114916</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <f aca="false">C13*A13</f>
         <v>0.428847974229833</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.285898649486555</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.214423987114916</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>15228.6786003336</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.0987646046427245</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">C14*A14</f>
         <v>0.296293813928173</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.131686139523633</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.0987646046427245</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>6674.12494574767</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.0432846032740143</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">C15*A15</f>
         <v>0.173138413096057</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.0577128043653524</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.0432846032740143</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="19" t="n">
         <v>1736.66497661918</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0112630277592767</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="13" t="n">
         <f aca="false">C16*A16</f>
         <v>0.0563151387963833</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.0150173703457022</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="13" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0112630277592767</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="23" t="n">
         <f aca="false">SUM(B11:B16)</f>
         <v>154191.662644958</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="24" t="n">
         <f aca="false">SUM(C11:C16)</f>
         <v>1</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="25" t="n">
         <f aca="false">SUM(D11:D16)</f>
         <v>1.30476270994767</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="25" t="n">
         <f aca="false">SUM(E11:E16)</f>
         <v>0.957204790250873</v>
       </c>
-      <c r="F17" s="24" t="n">
+      <c r="F17" s="26" t="n">
         <f aca="false">SUM(F11:F16)</f>
         <v>0.717903592688155</v>
       </c>
@@ -3685,16 +3693,16 @@
       <c r="A19" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <f aca="false">D17/E17</f>
         <v>1.3630967199879</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="27" t="n">
         <f aca="false">B19*60</f>
         <v>81.7858031992739</v>
       </c>
@@ -3781,19 +3789,19 @@
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="26" t="n">
+      <c r="E5" s="28" t="n">
         <v>1.41568125204773</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="28" t="n">
         <v>10.41706305183</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="29" t="n">
         <v>0.694470870122</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H5" s="16" t="n">
         <v>8.15401372730886</v>
       </c>
     </row>
@@ -3807,19 +3815,19 @@
       <c r="C6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="28" t="n">
         <v>1.40478117377424</v>
       </c>
-      <c r="F6" s="26" t="n">
+      <c r="F6" s="28" t="n">
         <v>10.3557644187949</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="29" t="n">
         <v>0.690384294586323</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="16" t="n">
         <v>8.1391259030073</v>
       </c>
     </row>
@@ -3833,19 +3841,19 @@
       <c r="C7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="28" t="n">
         <v>1.41112482199878</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="28" t="n">
         <v>10.3869468985734</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="29" t="n">
         <v>0.692463126571563</v>
       </c>
-      <c r="H7" s="15" t="n">
+      <c r="H7" s="16" t="n">
         <v>8.15133553167152</v>
       </c>
     </row>
@@ -3859,19 +3867,19 @@
       <c r="C8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E8" s="28" t="n">
         <v>1.41005154497534</v>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="28" t="n">
         <v>10.3882635073593</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="29" t="n">
         <v>0.692550900490619</v>
       </c>
-      <c r="H8" s="15" t="n">
+      <c r="H8" s="16" t="n">
         <v>8.14410345276529</v>
       </c>
     </row>
@@ -3885,49 +3893,49 @@
       <c r="C9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="26" t="n">
+      <c r="E9" s="28" t="n">
         <v>1.41506038197857</v>
       </c>
-      <c r="F9" s="26" t="n">
+      <c r="F9" s="28" t="n">
         <v>10.4180403658862</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="29" t="n">
         <v>0.694536024392415</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="16" t="n">
         <v>8.14967306104231</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="30" t="n">
         <f aca="false">AVERAGE(D5:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="25" t="n">
         <f aca="false">AVERAGE(E5:E9)</f>
         <v>1.41133983495493</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="25" t="n">
         <f aca="false">AVERAGE(F5:F9)</f>
         <v>10.3932156484888</v>
       </c>
-      <c r="G10" s="24" t="n">
+      <c r="G10" s="26" t="n">
         <f aca="false">AVERAGE(G5:G9)</f>
         <v>0.692881043232584</v>
       </c>
-      <c r="H10" s="25" t="n">
+      <c r="H10" s="27" t="n">
         <f aca="false">AVERAGE(H5:H9)</f>
         <v>8.14765033515906</v>
       </c>
@@ -3942,23 +3950,23 @@
       <c r="C11" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="31" t="n">
         <f aca="false">STDEV(D5:D9)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="13" t="n">
         <f aca="false">STDEV(E5:E9)</f>
         <v>0.00439921386882577</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <f aca="false">STDEV(F5:F9)</f>
         <v>0.0257457801048861</v>
       </c>
-      <c r="G11" s="30" t="n">
+      <c r="G11" s="32" t="n">
         <f aca="false">STDEV(G5:G9)</f>
         <v>0.00171638534032576</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="12" t="n">
         <f aca="false">STDEV(H5:H9)</f>
         <v>0.00598772016738544</v>
       </c>
@@ -3973,19 +3981,19 @@
       <c r="C13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="20" t="n">
         <v>2057</v>
       </c>
-      <c r="E13" s="26" t="n">
+      <c r="E13" s="28" t="n">
         <v>8.17396989080396</v>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="28" t="n">
         <v>3.99164297815367</v>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="29" t="n">
         <v>0.997910744538417</v>
       </c>
-      <c r="H13" s="15" t="n">
+      <c r="H13" s="16" t="n">
         <v>122.86624734036</v>
       </c>
     </row>
@@ -3999,19 +4007,19 @@
       <c r="C14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="20" t="n">
         <v>2322</v>
       </c>
-      <c r="E14" s="26" t="n">
+      <c r="E14" s="28" t="n">
         <v>8.36617034494946</v>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="28" t="n">
         <v>3.99796981609719</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="29" t="n">
         <v>0.999492454024297</v>
       </c>
-      <c r="H14" s="15" t="n">
+      <c r="H14" s="16" t="n">
         <v>125.556280759266</v>
       </c>
     </row>
@@ -4025,19 +4033,19 @@
       <c r="C15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="20" t="n">
         <v>2281</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="28" t="n">
         <v>8.43227902433431</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="28" t="n">
         <v>3.99856012486839</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="29" t="n">
         <v>0.999640031217098</v>
       </c>
-      <c r="H15" s="15" t="n">
+      <c r="H15" s="16" t="n">
         <v>126.529732118686</v>
       </c>
     </row>
@@ -4051,19 +4059,19 @@
       <c r="C16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="20" t="n">
         <v>2405</v>
       </c>
-      <c r="E16" s="26" t="n">
+      <c r="E16" s="28" t="n">
         <v>8.47594504973996</v>
       </c>
-      <c r="F16" s="26" t="n">
+      <c r="F16" s="28" t="n">
         <v>3.99656930819725</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="29" t="n">
         <v>0.999142327049313</v>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H16" s="16" t="n">
         <v>127.248313182336</v>
       </c>
     </row>
@@ -4077,49 +4085,49 @@
       <c r="C17" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="20" t="n">
         <v>2182</v>
       </c>
-      <c r="E17" s="26" t="n">
+      <c r="E17" s="28" t="n">
         <v>8.24549095686411</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="28" t="n">
         <v>3.98926368262925</v>
       </c>
-      <c r="G17" s="27" t="n">
+      <c r="G17" s="29" t="n">
         <v>0.997315920657312</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="16" t="n">
         <v>124.015231072863</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="28" t="n">
+      <c r="D18" s="30" t="n">
         <f aca="false">AVERAGE(D13:D17)</f>
         <v>2249.4</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="25" t="n">
         <f aca="false">AVERAGE(E13:E17)</f>
         <v>8.33877105333836</v>
       </c>
-      <c r="F18" s="23" t="n">
+      <c r="F18" s="25" t="n">
         <f aca="false">AVERAGE(F13:F17)</f>
         <v>3.99480118198915</v>
       </c>
-      <c r="G18" s="24" t="n">
+      <c r="G18" s="26" t="n">
         <f aca="false">AVERAGE(G13:G17)</f>
         <v>0.998700295497287</v>
       </c>
-      <c r="H18" s="25" t="n">
+      <c r="H18" s="27" t="n">
         <f aca="false">AVERAGE(H13:H17)</f>
         <v>125.243160894702</v>
       </c>
@@ -4134,23 +4142,23 @@
       <c r="C19" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="31" t="n">
         <f aca="false">STDEV(D13:D17)</f>
         <v>134.202458993865</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <f aca="false">STDEV(E13:E17)</f>
         <v>0.126660734523659</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="13" t="n">
         <f aca="false">STDEV(F13:F17)</f>
         <v>0.00412111376314653</v>
       </c>
-      <c r="G19" s="30" t="n">
+      <c r="G19" s="32" t="n">
         <f aca="false">STDEV(G13:G17)</f>
         <v>0.00103027844078667</v>
       </c>
-      <c r="H19" s="11" t="n">
+      <c r="H19" s="12" t="n">
         <f aca="false">STDEV(H13:H17)</f>
         <v>1.79801800274308</v>
       </c>
@@ -4165,19 +4173,19 @@
       <c r="C21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D21" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="E21" s="26" t="n">
+      <c r="E21" s="28" t="n">
         <v>1.92326099427399</v>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F21" s="28" t="n">
         <v>1.11835315374716</v>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G21" s="29" t="n">
         <v>0.838764865310369</v>
       </c>
-      <c r="H21" s="15" t="n">
+      <c r="H21" s="16" t="n">
         <v>103.183559924514</v>
       </c>
     </row>
@@ -4191,19 +4199,19 @@
       <c r="C22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="20" t="n">
         <v>132</v>
       </c>
-      <c r="E22" s="26" t="n">
+      <c r="E22" s="28" t="n">
         <v>2.19496828076005</v>
       </c>
-      <c r="F22" s="26" t="n">
+      <c r="F22" s="28" t="n">
         <v>1.16998792335286</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="29" t="n">
         <v>0.877490942514644</v>
       </c>
-      <c r="H22" s="15" t="n">
+      <c r="H22" s="16" t="n">
         <v>112.563637809349</v>
       </c>
     </row>
@@ -4217,19 +4225,19 @@
       <c r="C23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="20" t="n">
         <v>103</v>
       </c>
-      <c r="E23" s="26" t="n">
+      <c r="E23" s="28" t="n">
         <v>2.16919098238202</v>
       </c>
-      <c r="F23" s="26" t="n">
+      <c r="F23" s="28" t="n">
         <v>1.15695083320826</v>
       </c>
-      <c r="G23" s="27" t="n">
+      <c r="G23" s="29" t="n">
         <v>0.867713124906193</v>
       </c>
-      <c r="H23" s="15" t="n">
+      <c r="H23" s="16" t="n">
         <v>112.495237660193</v>
       </c>
     </row>
@@ -4243,19 +4251,19 @@
       <c r="C24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="20" t="n">
         <v>163</v>
       </c>
-      <c r="E24" s="26" t="n">
+      <c r="E24" s="28" t="n">
         <v>2.18299558493472</v>
       </c>
-      <c r="F24" s="26" t="n">
+      <c r="F24" s="28" t="n">
         <v>1.15878854510669</v>
       </c>
-      <c r="G24" s="27" t="n">
+      <c r="G24" s="29" t="n">
         <v>0.869091408830016</v>
       </c>
-      <c r="H24" s="15" t="n">
+      <c r="H24" s="16" t="n">
         <v>113.031610166654</v>
       </c>
     </row>
@@ -4269,49 +4277,49 @@
       <c r="C25" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D25" s="20" t="n">
         <v>146</v>
       </c>
-      <c r="E25" s="26" t="n">
+      <c r="E25" s="28" t="n">
         <v>2.18999027237302</v>
       </c>
-      <c r="F25" s="26" t="n">
+      <c r="F25" s="28" t="n">
         <v>1.16263319725305</v>
       </c>
-      <c r="G25" s="27" t="n">
+      <c r="G25" s="29" t="n">
         <v>0.871974897939787</v>
       </c>
-      <c r="H25" s="15" t="n">
+      <c r="H25" s="16" t="n">
         <v>113.018806492743</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D26" s="28" t="n">
+      <c r="D26" s="30" t="n">
         <f aca="false">AVERAGE(D21:D25)</f>
         <v>124.6</v>
       </c>
-      <c r="E26" s="23" t="n">
+      <c r="E26" s="25" t="n">
         <f aca="false">AVERAGE(E21:E25)</f>
         <v>2.13208122294476</v>
       </c>
-      <c r="F26" s="23" t="n">
+      <c r="F26" s="25" t="n">
         <f aca="false">AVERAGE(F21:F25)</f>
         <v>1.1533427305336</v>
       </c>
-      <c r="G26" s="24" t="n">
+      <c r="G26" s="26" t="n">
         <f aca="false">AVERAGE(G21:G25)</f>
         <v>0.865007047900202</v>
       </c>
-      <c r="H26" s="25" t="n">
+      <c r="H26" s="27" t="n">
         <f aca="false">AVERAGE(H21:H25)</f>
         <v>110.85857041069</v>
       </c>
@@ -4326,23 +4334,23 @@
       <c r="C27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="29" t="n">
+      <c r="D27" s="31" t="n">
         <f aca="false">STDEV(D21:D25)</f>
         <v>33.6645213837951</v>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="E27" s="13" t="n">
         <f aca="false">STDEV(E21:E25)</f>
         <v>0.11713617550825</v>
       </c>
-      <c r="F27" s="12" t="n">
+      <c r="F27" s="13" t="n">
         <f aca="false">STDEV(F21:F25)</f>
         <v>0.0201886168472803</v>
       </c>
-      <c r="G27" s="30" t="n">
+      <c r="G27" s="32" t="n">
         <f aca="false">STDEV(G21:G25)</f>
         <v>0.0151414626354602</v>
       </c>
-      <c r="H27" s="11" t="n">
+      <c r="H27" s="12" t="n">
         <f aca="false">STDEV(H21:H25)</f>
         <v>4.29768665079471</v>
       </c>
@@ -4357,19 +4365,19 @@
       <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="19" t="n">
+      <c r="D29" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="26" t="n">
+      <c r="E29" s="28" t="n">
         <v>1.39488508907472</v>
       </c>
-      <c r="F29" s="26" t="n">
+      <c r="F29" s="28" t="n">
         <v>10.3139826700539</v>
       </c>
-      <c r="G29" s="27" t="n">
+      <c r="G29" s="29" t="n">
         <v>0.687598844670258</v>
       </c>
-      <c r="H29" s="15" t="n">
+      <c r="H29" s="16" t="n">
         <v>8.11452840496641</v>
       </c>
     </row>
@@ -4383,19 +4391,19 @@
       <c r="C30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="26" t="n">
+      <c r="E30" s="28" t="n">
         <v>1.40656119390452</v>
       </c>
-      <c r="F30" s="26" t="n">
+      <c r="F30" s="28" t="n">
         <v>10.3630483811675</v>
       </c>
-      <c r="G30" s="27" t="n">
+      <c r="G30" s="29" t="n">
         <v>0.690869892077835</v>
       </c>
-      <c r="H30" s="15" t="n">
+      <c r="H30" s="16" t="n">
         <v>8.14371105201414</v>
       </c>
     </row>
@@ -4409,19 +4417,19 @@
       <c r="C31" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="26" t="n">
+      <c r="E31" s="28" t="n">
         <v>1.39854042505951</v>
       </c>
-      <c r="F31" s="26" t="n">
+      <c r="F31" s="28" t="n">
         <v>10.3285490305602</v>
       </c>
-      <c r="G31" s="27" t="n">
+      <c r="G31" s="29" t="n">
         <v>0.68856993537068</v>
       </c>
-      <c r="H31" s="15" t="n">
+      <c r="H31" s="16" t="n">
         <v>8.12431884239402</v>
       </c>
     </row>
@@ -4435,19 +4443,19 @@
       <c r="C32" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="26" t="n">
+      <c r="E32" s="28" t="n">
         <v>1.40824699461638</v>
       </c>
-      <c r="F32" s="26" t="n">
+      <c r="F32" s="28" t="n">
         <v>10.3729702387231</v>
       </c>
-      <c r="G32" s="27" t="n">
+      <c r="G32" s="29" t="n">
         <v>0.691531349248205</v>
       </c>
-      <c r="H32" s="15" t="n">
+      <c r="H32" s="16" t="n">
         <v>8.14567262147897</v>
       </c>
     </row>
@@ -4461,49 +4469,49 @@
       <c r="C33" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D33" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="26" t="n">
+      <c r="E33" s="28" t="n">
         <v>1.39539099827095</v>
       </c>
-      <c r="F33" s="26" t="n">
+      <c r="F33" s="28" t="n">
         <v>10.3085680685575</v>
       </c>
-      <c r="G33" s="27" t="n">
+      <c r="G33" s="29" t="n">
         <v>0.687237871237167</v>
       </c>
-      <c r="H33" s="15" t="n">
+      <c r="H33" s="16" t="n">
         <v>8.12173517596729</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D34" s="28" t="n">
+      <c r="D34" s="30" t="n">
         <f aca="false">AVERAGE(D29:D33)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="23" t="n">
+      <c r="E34" s="25" t="n">
         <f aca="false">AVERAGE(E29:E33)</f>
         <v>1.40072494018522</v>
       </c>
-      <c r="F34" s="23" t="n">
+      <c r="F34" s="25" t="n">
         <f aca="false">AVERAGE(F29:F33)</f>
         <v>10.3374236778124</v>
       </c>
-      <c r="G34" s="24" t="n">
+      <c r="G34" s="26" t="n">
         <f aca="false">AVERAGE(G29:G33)</f>
         <v>0.689161578520829</v>
       </c>
-      <c r="H34" s="25" t="n">
+      <c r="H34" s="27" t="n">
         <f aca="false">AVERAGE(H29:H33)</f>
         <v>8.12999321936416</v>
       </c>
@@ -4518,23 +4526,23 @@
       <c r="C35" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="29" t="n">
+      <c r="D35" s="31" t="n">
         <f aca="false">STDEV(D29:D33)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="12" t="n">
+      <c r="E35" s="13" t="n">
         <f aca="false">STDEV(E29:E33)</f>
         <v>0.00628430712197881</v>
       </c>
-      <c r="F35" s="12" t="n">
+      <c r="F35" s="13" t="n">
         <f aca="false">STDEV(F29:F33)</f>
         <v>0.0290734836606808</v>
       </c>
-      <c r="G35" s="30" t="n">
+      <c r="G35" s="32" t="n">
         <f aca="false">STDEV(G29:G33)</f>
         <v>0.00193823224404539</v>
       </c>
-      <c r="H35" s="11" t="n">
+      <c r="H35" s="12" t="n">
         <f aca="false">STDEV(H29:H33)</f>
         <v>0.0139066252411523</v>
       </c>
@@ -4549,19 +4557,19 @@
       <c r="C37" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="19" t="n">
+      <c r="D37" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="E37" s="26" t="n">
+      <c r="E37" s="28" t="n">
         <v>2.60866603726795</v>
       </c>
-      <c r="F37" s="26" t="n">
+      <c r="F37" s="28" t="n">
         <v>3.19126005156441</v>
       </c>
-      <c r="G37" s="27" t="n">
+      <c r="G37" s="29" t="n">
         <v>0.797815012891104</v>
       </c>
-      <c r="H37" s="15" t="n">
+      <c r="H37" s="16" t="n">
         <v>49.0464455127523</v>
       </c>
     </row>
@@ -4575,19 +4583,19 @@
       <c r="C38" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D38" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="E38" s="26" t="n">
+      <c r="E38" s="28" t="n">
         <v>2.82534499097601</v>
       </c>
-      <c r="F38" s="26" t="n">
+      <c r="F38" s="28" t="n">
         <v>3.30026829017066</v>
       </c>
-      <c r="G38" s="27" t="n">
+      <c r="G38" s="29" t="n">
         <v>0.825067072542664</v>
       </c>
-      <c r="H38" s="15" t="n">
+      <c r="H38" s="16" t="n">
         <v>51.3657328900963</v>
       </c>
     </row>
@@ -4601,19 +4609,19 @@
       <c r="C39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D39" s="19" t="n">
+      <c r="D39" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="E39" s="26" t="n">
+      <c r="E39" s="28" t="n">
         <v>2.85359245810866</v>
       </c>
-      <c r="F39" s="26" t="n">
+      <c r="F39" s="28" t="n">
         <v>3.28467263694278</v>
       </c>
-      <c r="G39" s="27" t="n">
+      <c r="G39" s="29" t="n">
         <v>0.821168159235695</v>
       </c>
-      <c r="H39" s="15" t="n">
+      <c r="H39" s="16" t="n">
         <v>52.1256047134971</v>
       </c>
     </row>
@@ -4627,19 +4635,19 @@
       <c r="C40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D40" s="19" t="n">
+      <c r="D40" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="E40" s="26" t="n">
+      <c r="E40" s="28" t="n">
         <v>3.09387009388168</v>
       </c>
-      <c r="F40" s="26" t="n">
+      <c r="F40" s="28" t="n">
         <v>3.33964538777848</v>
       </c>
-      <c r="G40" s="27" t="n">
+      <c r="G40" s="29" t="n">
         <v>0.834911346944621</v>
       </c>
-      <c r="H40" s="15" t="n">
+      <c r="H40" s="16" t="n">
         <v>55.5844061504932</v>
       </c>
     </row>
@@ -4653,49 +4661,49 @@
       <c r="C41" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D41" s="19" t="n">
+      <c r="D41" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="E41" s="26" t="n">
+      <c r="E41" s="28" t="n">
         <v>2.82902707642674</v>
       </c>
-      <c r="F41" s="26" t="n">
+      <c r="F41" s="28" t="n">
         <v>3.29777554828438</v>
       </c>
-      <c r="G41" s="27" t="n">
+      <c r="G41" s="29" t="n">
         <v>0.824443887071095</v>
       </c>
-      <c r="H41" s="15" t="n">
+      <c r="H41" s="16" t="n">
         <v>51.4715516869879</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D42" s="28" t="n">
+      <c r="D42" s="30" t="n">
         <f aca="false">AVERAGE(D37:D41)</f>
         <v>30</v>
       </c>
-      <c r="E42" s="23" t="n">
+      <c r="E42" s="25" t="n">
         <f aca="false">AVERAGE(E37:E41)</f>
         <v>2.84210013133221</v>
       </c>
-      <c r="F42" s="23" t="n">
+      <c r="F42" s="25" t="n">
         <f aca="false">AVERAGE(F37:F41)</f>
         <v>3.28272438294814</v>
       </c>
-      <c r="G42" s="24" t="n">
+      <c r="G42" s="26" t="n">
         <f aca="false">AVERAGE(G37:G41)</f>
         <v>0.820681095737036</v>
       </c>
-      <c r="H42" s="25" t="n">
+      <c r="H42" s="27" t="n">
         <f aca="false">AVERAGE(H37:H41)</f>
         <v>51.9187481907654</v>
       </c>
@@ -4710,23 +4718,23 @@
       <c r="C43" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D43" s="29" t="n">
+      <c r="D43" s="31" t="n">
         <f aca="false">STDEV(D37:D41)</f>
         <v>9</v>
       </c>
-      <c r="E43" s="12" t="n">
+      <c r="E43" s="13" t="n">
         <f aca="false">STDEV(E37:E41)</f>
         <v>0.172092492123722</v>
       </c>
-      <c r="F43" s="12" t="n">
+      <c r="F43" s="13" t="n">
         <f aca="false">STDEV(F37:F41)</f>
         <v>0.0550995613834784</v>
       </c>
-      <c r="G43" s="30" t="n">
+      <c r="G43" s="32" t="n">
         <f aca="false">STDEV(G37:G41)</f>
         <v>0.0137748903458695</v>
       </c>
-      <c r="H43" s="11" t="n">
+      <c r="H43" s="12" t="n">
         <f aca="false">STDEV(H37:H41)</f>
         <v>2.3577410379746</v>
       </c>
@@ -4741,19 +4749,19 @@
       <c r="C45" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="19" t="n">
+      <c r="D45" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="E45" s="26" t="n">
+      <c r="E45" s="28" t="n">
         <v>1.30476270994767</v>
       </c>
-      <c r="F45" s="26" t="n">
+      <c r="F45" s="28" t="n">
         <v>0.957204790250873</v>
       </c>
-      <c r="G45" s="27" t="n">
+      <c r="G45" s="29" t="n">
         <v>0.717903592688155</v>
       </c>
-      <c r="H45" s="15" t="n">
+      <c r="H45" s="16" t="n">
         <v>81.7858031992739</v>
       </c>
     </row>
@@ -4767,19 +4775,19 @@
       <c r="C46" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D46" s="19" t="n">
+      <c r="D46" s="20" t="n">
         <v>32</v>
       </c>
-      <c r="E46" s="26" t="n">
+      <c r="E46" s="28" t="n">
         <v>1.3751723417863</v>
       </c>
-      <c r="F46" s="26" t="n">
+      <c r="F46" s="28" t="n">
         <v>0.975368869097814</v>
       </c>
-      <c r="G46" s="27" t="n">
+      <c r="G46" s="29" t="n">
         <v>0.731526651823361</v>
       </c>
-      <c r="H46" s="15" t="n">
+      <c r="H46" s="16" t="n">
         <v>84.5939860511415</v>
       </c>
     </row>
@@ -4793,19 +4801,19 @@
       <c r="C47" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D47" s="19" t="n">
+      <c r="D47" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="E47" s="26" t="n">
+      <c r="E47" s="28" t="n">
         <v>1.39335862489791</v>
       </c>
-      <c r="F47" s="26" t="n">
+      <c r="F47" s="28" t="n">
         <v>0.970303494294256</v>
       </c>
-      <c r="G47" s="27" t="n">
+      <c r="G47" s="29" t="n">
         <v>0.727727620720692</v>
       </c>
-      <c r="H47" s="15" t="n">
+      <c r="H47" s="16" t="n">
         <v>86.1601735802068</v>
       </c>
     </row>
@@ -4819,19 +4827,19 @@
       <c r="C48" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D48" s="19" t="n">
+      <c r="D48" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="E48" s="26" t="n">
+      <c r="E48" s="28" t="n">
         <v>1.38930425101755</v>
       </c>
-      <c r="F48" s="26" t="n">
+      <c r="F48" s="28" t="n">
         <v>0.972201327156678</v>
       </c>
-      <c r="G48" s="27" t="n">
+      <c r="G48" s="29" t="n">
         <v>0.729150995367509</v>
       </c>
-      <c r="H48" s="15" t="n">
+      <c r="H48" s="16" t="n">
         <v>85.7417622591037</v>
       </c>
     </row>
@@ -4845,49 +4853,49 @@
       <c r="C49" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D49" s="19" t="n">
+      <c r="D49" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="E49" s="26" t="n">
+      <c r="E49" s="28" t="n">
         <v>1.48083520571888</v>
       </c>
-      <c r="F49" s="26" t="n">
+      <c r="F49" s="28" t="n">
         <v>0.995720294714835</v>
       </c>
-      <c r="G49" s="27" t="n">
+      <c r="G49" s="29" t="n">
         <v>0.746790221036126</v>
       </c>
-      <c r="H49" s="15" t="n">
+      <c r="H49" s="16" t="n">
         <v>89.2319990008625</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="13" t="s">
+      <c r="A50" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B50" s="13" t="s">
+      <c r="B50" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="13" t="s">
+      <c r="C50" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D50" s="28" t="n">
+      <c r="D50" s="30" t="n">
         <f aca="false">AVERAGE(D45:D49)</f>
         <v>28.6</v>
       </c>
-      <c r="E50" s="23" t="n">
+      <c r="E50" s="25" t="n">
         <f aca="false">AVERAGE(E45:E49)</f>
         <v>1.38868662667366</v>
       </c>
-      <c r="F50" s="23" t="n">
+      <c r="F50" s="25" t="n">
         <f aca="false">AVERAGE(F45:F49)</f>
         <v>0.974159755102891</v>
       </c>
-      <c r="G50" s="24" t="n">
+      <c r="G50" s="26" t="n">
         <f aca="false">AVERAGE(G45:G49)</f>
         <v>0.730619816327168</v>
       </c>
-      <c r="H50" s="25" t="n">
+      <c r="H50" s="27" t="n">
         <f aca="false">AVERAGE(H45:H49)</f>
         <v>85.5027448181177</v>
       </c>
@@ -4902,23 +4910,23 @@
       <c r="C51" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D51" s="29" t="n">
+      <c r="D51" s="31" t="n">
         <f aca="false">STDEV(D45:D49)</f>
         <v>8.01872807869178</v>
       </c>
-      <c r="E51" s="12" t="n">
+      <c r="E51" s="13" t="n">
         <f aca="false">STDEV(E45:E49)</f>
         <v>0.0627284412008175</v>
       </c>
-      <c r="F51" s="12" t="n">
+      <c r="F51" s="13" t="n">
         <f aca="false">STDEV(F45:F49)</f>
         <v>0.0138969047416033</v>
       </c>
-      <c r="G51" s="30" t="n">
+      <c r="G51" s="32" t="n">
         <f aca="false">STDEV(G45:G49)</f>
         <v>0.0104226785562025</v>
       </c>
-      <c r="H51" s="11" t="n">
+      <c r="H51" s="12" t="n">
         <f aca="false">STDEV(H45:H49)</f>
         <v>2.69435410480351</v>
       </c>

</xml_diff>

<commit_message>
Ajusta o acabamento da planilha do T2
Impressão em paisagem cabendo na largura da página, alinhamento do ∞ e
das variações, coluna de destino do roteamento mais larga e rótulo da
conferência de tempos sem corte. Os valores não mudam (410 fórmulas,
sem erros; 60 células da comparação conferidas contra o analise_indices.py).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/T2 - Avaliação de Aprendizagem/indices_desempenho.xlsx
+++ b/T2 - Avaliação de Aprendizagem/indices_desempenho.xlsx
@@ -219,7 +219,7 @@
     <t xml:space="preserve">W (minutos)</t>
   </si>
   <si>
-    <t xml:space="preserve">Conferência: soma dos tempos = tempo global?</t>
+    <t xml:space="preserve">Soma dos tempos = tempo global?</t>
   </si>
   <si>
     <t xml:space="preserve">Atual - Q2 (N2 - Especialista)</t>
@@ -386,7 +386,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -407,8 +407,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -429,6 +429,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -457,6 +461,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -769,7 +777,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1307,7 +1315,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1318,14 +1326,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:M24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="11"/>
@@ -1402,30 +1409,30 @@
       <c r="E5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="13" t="n">
         <f aca="false">(G5+H5)/2</f>
         <v>8</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="14" t="n">
         <f aca="false">60/I5</f>
         <v>7.5</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="M5" s="11" t="n">
+      <c r="M5" s="12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1445,20 +1452,20 @@
       <c r="E6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="13" t="n">
         <f aca="false">(G6+H6)/2</f>
         <v>30</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="14" t="n">
         <f aca="false">60/I6</f>
         <v>2</v>
       </c>
@@ -1479,20 +1486,20 @@
       <c r="E7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="13" t="n">
         <f aca="false">(G7+H7)/2</f>
         <v>45</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="14" t="n">
         <f aca="false">60/I7</f>
         <v>1.33333333333333</v>
       </c>
@@ -1513,30 +1520,30 @@
       <c r="E9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="H9" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="13" t="n">
         <f aca="false">(G9+H9)/2</f>
         <v>8</v>
       </c>
-      <c r="J9" s="13" t="n">
+      <c r="J9" s="14" t="n">
         <f aca="false">60/I9</f>
         <v>7.5</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="K9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="L9" s="11" t="n">
+      <c r="L9" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="M9" s="11" t="n">
+      <c r="M9" s="12" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1556,20 +1563,20 @@
       <c r="E10" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="13" t="n">
         <f aca="false">(G10+H10)/2</f>
         <v>30</v>
       </c>
-      <c r="J10" s="13" t="n">
+      <c r="J10" s="14" t="n">
         <f aca="false">60/I10</f>
         <v>2</v>
       </c>
@@ -1590,26 +1597,26 @@
       <c r="E11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="13" t="n">
         <f aca="false">(G11+H11)/2</f>
         <v>45</v>
       </c>
-      <c r="J11" s="13" t="n">
+      <c r="J11" s="14" t="n">
         <f aca="false">60/I11</f>
         <v>1.33333333333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1634,10 +1641,10 @@
       <c r="B16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="16" t="n">
         <v>0.45</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="16" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1648,11 +1655,11 @@
       <c r="B17" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="13" t="n">
         <f aca="false">1-SUM(C16)</f>
         <v>0.55</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="13" t="n">
         <f aca="false">1-SUM(D16)</f>
         <v>0.7</v>
       </c>
@@ -1664,10 +1671,10 @@
       <c r="B18" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="17" t="n">
         <v>0.3</v>
       </c>
-      <c r="D18" s="16" t="n">
+      <c r="D18" s="17" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1678,10 +1685,10 @@
       <c r="B19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="16" t="n">
+      <c r="C19" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="D19" s="16" t="n">
+      <c r="D19" s="17" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -1692,11 +1699,11 @@
       <c r="B20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <f aca="false">1-SUM(C18:C19)</f>
         <v>0.6</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <f aca="false">1-SUM(D18:D19)</f>
         <v>0.6</v>
       </c>
@@ -1708,10 +1715,10 @@
       <c r="B21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="16" t="n">
+      <c r="C21" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="D21" s="16" t="n">
+      <c r="D21" s="17" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1722,11 +1729,11 @@
       <c r="B22" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="13" t="n">
         <f aca="false">1-SUM(C21)</f>
         <v>0.8</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="13" t="n">
         <f aca="false">1-SUM(D21)</f>
         <v>0.8</v>
       </c>
@@ -1739,7 +1746,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1750,7 +1757,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1779,7 +1786,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <f aca="false">Parâmetros!$E$5</f>
         <v>2</v>
       </c>
@@ -1788,7 +1795,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="17" t="str">
+      <c r="B5" s="19" t="str">
         <f aca="false">Parâmetros!$F$5</f>
         <v>∞</v>
       </c>
@@ -1797,7 +1804,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Parâmetros!$J$5</f>
         <v>7.5</v>
       </c>
@@ -1806,7 +1813,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="21" t="n">
         <v>146269.717459168</v>
       </c>
     </row>
@@ -1814,7 +1821,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1839,146 +1846,146 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="21" t="n">
         <v>1799.95110185165</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.0123056989041776</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>85779.4168018978</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.586446861947644</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">C12*A12</f>
         <v>0.586446861947644</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>4.39835146460733</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.293223430973822</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="21" t="n">
         <v>54849.1453557126</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.374986335575742</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">C13*A13</f>
         <v>0.749972671151484</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>5.62479503363613</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.374986335575742</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>3771.2275628848</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.025782695341143</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">C14*A14</f>
         <v>0.077348086023429</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.386740430117145</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.025782695341143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="21" t="n">
         <v>69.9766368214041</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.00047840823129325</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">C15*A15</f>
         <v>0.001913632925173</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.00717612346939875</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.00047840823129325</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="25" t="n">
         <f aca="false">SUM(B11:B15)</f>
         <v>146269.717459168</v>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C16" s="26" t="n">
         <f aca="false">SUM(C11:C15)</f>
         <v>1</v>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D16" s="27" t="n">
         <f aca="false">SUM(D11:D15)</f>
         <v>1.41568125204773</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="27" t="n">
         <f aca="false">SUM(E11:E15)</f>
         <v>10.41706305183</v>
       </c>
-      <c r="F16" s="26" t="n">
+      <c r="F16" s="28" t="n">
         <f aca="false">SUM(F11:F15)</f>
         <v>0.694470870122</v>
       </c>
@@ -1987,16 +1994,16 @@
       <c r="A18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="14" t="n">
         <f aca="false">D16/E16</f>
         <v>0.135900228788481</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="27" t="n">
+      <c r="B19" s="29" t="n">
         <f aca="false">B18*60</f>
         <v>8.15401372730886</v>
       </c>
@@ -2013,7 +2020,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2024,7 +2031,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2053,7 +2060,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <f aca="false">Parâmetros!$E$6</f>
         <v>2</v>
       </c>
@@ -2062,7 +2069,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="19" t="n">
         <f aca="false">Parâmetros!$F$6</f>
         <v>10</v>
       </c>
@@ -2071,7 +2078,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Parâmetros!$J$6</f>
         <v>2</v>
       </c>
@@ -2080,7 +2087,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="21" t="n">
         <v>146269.717459168</v>
       </c>
     </row>
@@ -2088,7 +2095,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>2057</v>
       </c>
     </row>
@@ -2113,290 +2120,290 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="21" t="n">
         <v>68.9358042832464</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.000471292386973333</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>473.318003565073</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.00323592614921952</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">C12*A12</f>
         <v>0.00323592614921952</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.00647185229843903</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.00161796307460976</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="21" t="n">
         <v>998.020987044089</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.00682315522570617</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">C13*A13</f>
         <v>0.0136463104514123</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.0272926209028247</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.00682315522570617</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>1917.09665392619</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.0131065861562312</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">C14*A14</f>
         <v>0.0393197584686936</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.0524263446249248</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.0131065861562312</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="21" t="n">
         <v>3102.75989075005</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.0212125923577872</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">C15*A15</f>
         <v>0.0848503694311489</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.0848503694311489</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.0212125923577872</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="21" t="n">
         <v>5724.31662190985</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0391353502375351</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">C16*A16</f>
         <v>0.195676751187675</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.15654140095014</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0391353502375351</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="B17" s="19" t="n">
+      <c r="B17" s="21" t="n">
         <v>9481.77895309404</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="24" t="n">
         <f aca="false">B17/$B$7</f>
         <v>0.064823937024018</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="14" t="n">
         <f aca="false">C17*A17</f>
         <v>0.388943622144108</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="14" t="n">
         <f aca="false">C17*MIN(A17,$B$4)*$B$6</f>
         <v>0.259295748096072</v>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="14" t="n">
         <f aca="false">C17*MIN(A17,$B$4)/$B$4</f>
         <v>0.064823937024018</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B18" s="19" t="n">
+      <c r="B18" s="21" t="n">
         <v>16807.0212294292</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="24" t="n">
         <f aca="false">B18/$B$7</f>
         <v>0.114904311851979</v>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="14" t="n">
         <f aca="false">C18*A18</f>
         <v>0.804330182963855</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="14" t="n">
         <f aca="false">C18*MIN(A18,$B$4)*$B$6</f>
         <v>0.459617247407917</v>
       </c>
-      <c r="F18" s="13" t="n">
+      <c r="F18" s="14" t="n">
         <f aca="false">C18*MIN(A18,$B$4)/$B$4</f>
         <v>0.114904311851979</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B19" s="19" t="n">
+      <c r="B19" s="21" t="n">
         <v>30899.1502329391</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="24" t="n">
         <f aca="false">B19/$B$7</f>
         <v>0.211247760436569</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="14" t="n">
         <f aca="false">C19*A19</f>
         <v>1.68998208349255</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">C19*MIN(A19,$B$4)*$B$6</f>
         <v>0.844991041746277</v>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="F19" s="14" t="n">
         <f aca="false">C19*MIN(A19,$B$4)/$B$4</f>
         <v>0.211247760436569</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="B20" s="19" t="n">
+      <c r="B20" s="21" t="n">
         <v>43355.2211746937</v>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C20" s="24" t="n">
         <f aca="false">B20/$B$7</f>
         <v>0.296405995224517</v>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="14" t="n">
         <f aca="false">C20*A20</f>
         <v>2.66765395702065</v>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="14" t="n">
         <f aca="false">C20*MIN(A20,$B$4)*$B$6</f>
         <v>1.18562398089807</v>
       </c>
-      <c r="F20" s="13" t="n">
+      <c r="F20" s="14" t="n">
         <f aca="false">C20*MIN(A20,$B$4)/$B$4</f>
         <v>0.296405995224517</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="21" t="n">
         <v>33442.0979075339</v>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="24" t="n">
         <f aca="false">B21/$B$7</f>
         <v>0.228633092949464</v>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="14" t="n">
         <f aca="false">C21*A21</f>
         <v>2.28633092949464</v>
       </c>
-      <c r="E21" s="13" t="n">
+      <c r="E21" s="14" t="n">
         <f aca="false">C21*MIN(A21,$B$4)*$B$6</f>
         <v>0.914532371797856</v>
       </c>
-      <c r="F21" s="13" t="n">
+      <c r="F21" s="14" t="n">
         <f aca="false">C21*MIN(A21,$B$4)/$B$4</f>
         <v>0.228633092949464</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="23" t="n">
+      <c r="B22" s="25" t="n">
         <f aca="false">SUM(B11:B21)</f>
         <v>146269.717459168</v>
       </c>
-      <c r="C22" s="24" t="n">
+      <c r="C22" s="26" t="n">
         <f aca="false">SUM(C11:C21)</f>
         <v>1</v>
       </c>
-      <c r="D22" s="25" t="n">
+      <c r="D22" s="27" t="n">
         <f aca="false">SUM(D11:D21)</f>
         <v>8.17396989080396</v>
       </c>
-      <c r="E22" s="25" t="n">
+      <c r="E22" s="27" t="n">
         <f aca="false">SUM(E11:E21)</f>
         <v>3.99164297815367</v>
       </c>
-      <c r="F22" s="26" t="n">
+      <c r="F22" s="28" t="n">
         <f aca="false">SUM(F11:F21)</f>
         <v>0.997910744538417</v>
       </c>
@@ -2405,16 +2412,16 @@
       <c r="A24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="14" t="n">
         <f aca="false">D22/E22</f>
         <v>2.04777078900599</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="27" t="n">
+      <c r="B25" s="29" t="n">
         <f aca="false">B24*60</f>
         <v>122.866247340359</v>
       </c>
@@ -2431,7 +2438,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2442,7 +2449,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2471,7 +2478,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <f aca="false">Parâmetros!$E$7</f>
         <v>1</v>
       </c>
@@ -2480,7 +2487,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="19" t="n">
         <f aca="false">Parâmetros!$F$7</f>
         <v>5</v>
       </c>
@@ -2489,7 +2496,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Parâmetros!$J$7</f>
         <v>1.33333333333333</v>
       </c>
@@ -2498,7 +2505,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="21" t="n">
         <v>146269.717459168</v>
       </c>
     </row>
@@ -2506,7 +2513,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>79</v>
       </c>
     </row>
@@ -2531,170 +2538,170 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="21" t="n">
         <v>23583.8175955433</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.161235134689631</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>41758.0095335674</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.285486362173525</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">C12*A12</f>
         <v>0.285486362173525</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.380648482898034</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.285486362173525</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="21" t="n">
         <v>33814.2295845244</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.231177240046039</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">C13*A13</f>
         <v>0.462354480092077</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.308236320061385</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.231177240046039</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>23065.2667063912</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.15768996554485</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">C14*A14</f>
         <v>0.473069896634551</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.210253287393134</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.15768996554485</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="21" t="n">
         <v>17509.3967848048</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.119706232355939</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">C15*A15</f>
         <v>0.478824929423756</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.159608309807919</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.119706232355939</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="21" t="n">
         <v>6538.99725433718</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0447050651900149</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">C16*A16</f>
         <v>0.223525325950075</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.0596067535866866</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0447050651900149</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="25" t="n">
         <f aca="false">SUM(B11:B16)</f>
         <v>146269.717459168</v>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="26" t="n">
         <f aca="false">SUM(C11:C16)</f>
         <v>1</v>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="27" t="n">
         <f aca="false">SUM(D11:D16)</f>
         <v>1.92326099427398</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="27" t="n">
         <f aca="false">SUM(E11:E16)</f>
         <v>1.11835315374716</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="28" t="n">
         <f aca="false">SUM(F11:F16)</f>
         <v>0.838764865310368</v>
       </c>
@@ -2703,16 +2710,16 @@
       <c r="A19" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="14" t="n">
         <f aca="false">D17/E17</f>
         <v>1.7197259987419</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="27" t="n">
+      <c r="B20" s="29" t="n">
         <f aca="false">B19*60</f>
         <v>103.183559924514</v>
       </c>
@@ -2729,7 +2736,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2740,7 +2747,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2769,7 +2776,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <f aca="false">Parâmetros!$E$9</f>
         <v>2</v>
       </c>
@@ -2778,7 +2785,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="17" t="str">
+      <c r="B5" s="19" t="str">
         <f aca="false">Parâmetros!$F$9</f>
         <v>∞</v>
       </c>
@@ -2787,7 +2794,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Parâmetros!$J$9</f>
         <v>7.5</v>
       </c>
@@ -2796,7 +2803,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="21" t="n">
         <v>154191.662644958</v>
       </c>
     </row>
@@ -2804,7 +2811,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2829,146 +2836,146 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="21" t="n">
         <v>1939.06857775338</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.0125757031508136</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>92461.1699494906</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.599650904357856</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">C12*A12</f>
         <v>0.599650904357856</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>4.49738178268392</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.299825452178928</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="21" t="n">
         <v>56785.0519056795</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.368275761034063</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">C13*A13</f>
         <v>0.736551522068127</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>5.52413641551095</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.368275761034063</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>2977.11152589601</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.0193078631803271</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">C14*A14</f>
         <v>0.0579235895409813</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.289617947704907</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.0193078631803271</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="21" t="n">
         <v>29.2606861386448</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.000189768276939983</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">C15*A15</f>
         <v>0.000759073107759931</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.00284652415409974</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.000189768276939983</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="25" t="n">
         <f aca="false">SUM(B11:B15)</f>
         <v>154191.662644958</v>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C16" s="26" t="n">
         <f aca="false">SUM(C11:C15)</f>
         <v>1</v>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D16" s="27" t="n">
         <f aca="false">SUM(D11:D15)</f>
         <v>1.39488508907472</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="27" t="n">
         <f aca="false">SUM(E11:E15)</f>
         <v>10.3139826700539</v>
       </c>
-      <c r="F16" s="26" t="n">
+      <c r="F16" s="28" t="n">
         <f aca="false">SUM(F11:F15)</f>
         <v>0.687598844670259</v>
       </c>
@@ -2977,16 +2984,16 @@
       <c r="A18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="14" t="n">
         <f aca="false">D16/E16</f>
         <v>0.135242140082773</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="27" t="n">
+      <c r="B19" s="29" t="n">
         <f aca="false">B18*60</f>
         <v>8.11452840496641</v>
       </c>
@@ -3003,7 +3010,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3014,7 +3021,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3043,7 +3050,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <f aca="false">Parâmetros!$E$10</f>
         <v>2</v>
       </c>
@@ -3052,7 +3059,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="19" t="n">
         <f aca="false">Parâmetros!$F$10</f>
         <v>10</v>
       </c>
@@ -3061,7 +3068,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Parâmetros!$J$10</f>
         <v>2</v>
       </c>
@@ -3070,7 +3077,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="21" t="n">
         <v>154191.662644958</v>
       </c>
     </row>
@@ -3078,7 +3085,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3103,290 +3110,290 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="21" t="n">
         <v>13755.7628458915</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.0892121053105547</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>34838.9529565573</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.225945763596683</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">C12*A12</f>
         <v>0.225945763596683</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.451891527193367</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.112972881798342</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="21" t="n">
         <v>37189.4851482725</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.241189987255699</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">C13*A13</f>
         <v>0.482379974511398</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.964759949022796</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.241189987255699</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>28872.3286273032</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.187249609557585</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">C14*A14</f>
         <v>0.561748828672754</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.748998438230339</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.187249609557585</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="21" t="n">
         <v>17039.0442472659</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.110505613306084</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">C15*A15</f>
         <v>0.442022453224336</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.442022453224336</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.110505613306084</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="21" t="n">
         <v>9475.65576402098</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0614537491942067</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">C16*A16</f>
         <v>0.307268745971033</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.245814996776827</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0614537491942067</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="B17" s="19" t="n">
+      <c r="B17" s="21" t="n">
         <v>5719.80337375123</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="24" t="n">
         <f aca="false">B17/$B$7</f>
         <v>0.0370954127845528</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="14" t="n">
         <f aca="false">C17*A17</f>
         <v>0.222572476707317</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="14" t="n">
         <f aca="false">C17*MIN(A17,$B$4)*$B$6</f>
         <v>0.148381651138211</v>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="14" t="n">
         <f aca="false">C17*MIN(A17,$B$4)/$B$4</f>
         <v>0.0370954127845528</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B18" s="19" t="n">
+      <c r="B18" s="21" t="n">
         <v>3614.86460275762</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="24" t="n">
         <f aca="false">B18/$B$7</f>
         <v>0.0234439692830942</v>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="14" t="n">
         <f aca="false">C18*A18</f>
         <v>0.164107784981659</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="14" t="n">
         <f aca="false">C18*MIN(A18,$B$4)*$B$6</f>
         <v>0.0937758771323767</v>
       </c>
-      <c r="F18" s="13" t="n">
+      <c r="F18" s="14" t="n">
         <f aca="false">C18*MIN(A18,$B$4)/$B$4</f>
         <v>0.0234439692830942</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B19" s="19" t="n">
+      <c r="B19" s="21" t="n">
         <v>2269.19500326645</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="24" t="n">
         <f aca="false">B19/$B$7</f>
         <v>0.014716716613216</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="14" t="n">
         <f aca="false">C19*A19</f>
         <v>0.117733732905728</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">C19*MIN(A19,$B$4)*$B$6</f>
         <v>0.0588668664528639</v>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="F19" s="14" t="n">
         <f aca="false">C19*MIN(A19,$B$4)/$B$4</f>
         <v>0.014716716613216</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="B20" s="19" t="n">
+      <c r="B20" s="21" t="n">
         <v>1076.94461905677</v>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C20" s="24" t="n">
         <f aca="false">B20/$B$7</f>
         <v>0.00698445428619927</v>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="14" t="n">
         <f aca="false">C20*A20</f>
         <v>0.0628600885757934</v>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="14" t="n">
         <f aca="false">C20*MIN(A20,$B$4)*$B$6</f>
         <v>0.0279378171447971</v>
       </c>
-      <c r="F20" s="13" t="n">
+      <c r="F20" s="14" t="n">
         <f aca="false">C20*MIN(A20,$B$4)/$B$4</f>
         <v>0.00698445428619927</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="21" t="n">
         <v>339.625456814654</v>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="24" t="n">
         <f aca="false">B21/$B$7</f>
         <v>0.00220261881212525</v>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="14" t="n">
         <f aca="false">C21*A21</f>
         <v>0.0220261881212525</v>
       </c>
-      <c r="E21" s="13" t="n">
+      <c r="E21" s="14" t="n">
         <f aca="false">C21*MIN(A21,$B$4)*$B$6</f>
         <v>0.00881047524850098</v>
       </c>
-      <c r="F21" s="13" t="n">
+      <c r="F21" s="14" t="n">
         <f aca="false">C21*MIN(A21,$B$4)/$B$4</f>
         <v>0.00220261881212525</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="23" t="n">
+      <c r="B22" s="25" t="n">
         <f aca="false">SUM(B11:B21)</f>
         <v>154191.662644958</v>
       </c>
-      <c r="C22" s="24" t="n">
+      <c r="C22" s="26" t="n">
         <f aca="false">SUM(C11:C21)</f>
         <v>1</v>
       </c>
-      <c r="D22" s="25" t="n">
+      <c r="D22" s="27" t="n">
         <f aca="false">SUM(D11:D21)</f>
         <v>2.60866603726796</v>
       </c>
-      <c r="E22" s="25" t="n">
+      <c r="E22" s="27" t="n">
         <f aca="false">SUM(E11:E21)</f>
         <v>3.19126005156441</v>
       </c>
-      <c r="F22" s="26" t="n">
+      <c r="F22" s="28" t="n">
         <f aca="false">SUM(F11:F21)</f>
         <v>0.797815012891104</v>
       </c>
@@ -3395,16 +3402,16 @@
       <c r="A24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="14" t="n">
         <f aca="false">D22/E22</f>
         <v>0.817440758545873</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="27" t="n">
+      <c r="B25" s="29" t="n">
         <f aca="false">B24*60</f>
         <v>49.0464455127524</v>
       </c>
@@ -3421,7 +3428,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3432,7 +3439,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3461,7 +3468,7 @@
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <f aca="false">Parâmetros!$E$11</f>
         <v>1</v>
       </c>
@@ -3470,7 +3477,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="19" t="n">
         <f aca="false">Parâmetros!$F$11</f>
         <v>5</v>
       </c>
@@ -3479,7 +3486,7 @@
       <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="20" t="n">
         <f aca="false">Parâmetros!$J$11</f>
         <v>1.33333333333333</v>
       </c>
@@ -3488,7 +3495,7 @@
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="21" t="n">
         <v>154191.662644958</v>
       </c>
     </row>
@@ -3496,7 +3503,7 @@
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3521,170 +3528,170 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="21" t="n">
         <v>43496.9140695827</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">B11/$B$7</f>
         <v>0.282096407311845</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <f aca="false">C11*A11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)*$B$6</f>
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">C11*MIN(A11,$B$4)/$B$4</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>53992.8889684649</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">B12/$B$7</f>
         <v>0.350167369897223</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <f aca="false">C12*A12</f>
         <v>0.350167369897223</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)*$B$6</f>
         <v>0.466889826529631</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <f aca="false">C12*MIN(A12,$B$4)/$B$4</f>
         <v>0.350167369897223</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="21" t="n">
         <v>33062.39108421</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">B13/$B$7</f>
         <v>0.214423987114916</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <f aca="false">C13*A13</f>
         <v>0.428847974229833</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)*$B$6</f>
         <v>0.285898649486555</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <f aca="false">C13*MIN(A13,$B$4)/$B$4</f>
         <v>0.214423987114916</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>15228.6786003336</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">B14/$B$7</f>
         <v>0.0987646046427245</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <f aca="false">C14*A14</f>
         <v>0.296293813928173</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)*$B$6</f>
         <v>0.131686139523633</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <f aca="false">C14*MIN(A14,$B$4)/$B$4</f>
         <v>0.0987646046427245</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="21" t="n">
         <v>6674.12494574767</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">B15/$B$7</f>
         <v>0.0432846032740143</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <f aca="false">C15*A15</f>
         <v>0.173138413096057</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)*$B$6</f>
         <v>0.0577128043653524</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <f aca="false">C15*MIN(A15,$B$4)/$B$4</f>
         <v>0.0432846032740143</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="21" t="n">
         <v>1736.66497661918</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="24" t="n">
         <f aca="false">B16/$B$7</f>
         <v>0.0112630277592767</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">C16*A16</f>
         <v>0.0563151387963833</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)*$B$6</f>
         <v>0.0150173703457022</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="14" t="n">
         <f aca="false">C16*MIN(A16,$B$4)/$B$4</f>
         <v>0.0112630277592767</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="25" t="n">
         <f aca="false">SUM(B11:B16)</f>
         <v>154191.662644958</v>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="26" t="n">
         <f aca="false">SUM(C11:C16)</f>
         <v>1</v>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="27" t="n">
         <f aca="false">SUM(D11:D16)</f>
         <v>1.30476270994767</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="27" t="n">
         <f aca="false">SUM(E11:E16)</f>
         <v>0.957204790250873</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="28" t="n">
         <f aca="false">SUM(F11:F16)</f>
         <v>0.717903592688155</v>
       </c>
@@ -3693,16 +3700,16 @@
       <c r="A19" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="14" t="n">
         <f aca="false">D17/E17</f>
         <v>1.3630967199879</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="27" t="n">
+      <c r="B20" s="29" t="n">
         <f aca="false">B19*60</f>
         <v>81.7858031992739</v>
       </c>
@@ -3719,7 +3726,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3730,7 +3737,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3789,19 +3796,19 @@
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E5" s="30" t="n">
         <v>1.41568125204773</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="30" t="n">
         <v>10.41706305183</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="31" t="n">
         <v>0.694470870122</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <v>8.15401372730886</v>
       </c>
     </row>
@@ -3815,19 +3822,19 @@
       <c r="C6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="30" t="n">
         <v>1.40478117377424</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="30" t="n">
         <v>10.3557644187949</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="31" t="n">
         <v>0.690384294586323</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>8.1391259030073</v>
       </c>
     </row>
@@ -3841,19 +3848,19 @@
       <c r="C7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="30" t="n">
         <v>1.41112482199878</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="30" t="n">
         <v>10.3869468985734</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="31" t="n">
         <v>0.692463126571563</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <v>8.15133553167152</v>
       </c>
     </row>
@@ -3867,19 +3874,19 @@
       <c r="C8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="30" t="n">
         <v>1.41005154497534</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="30" t="n">
         <v>10.3882635073593</v>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="31" t="n">
         <v>0.692550900490619</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="17" t="n">
         <v>8.14410345276529</v>
       </c>
     </row>
@@ -3893,49 +3900,49 @@
       <c r="C9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="30" t="n">
         <v>1.41506038197857</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="30" t="n">
         <v>10.4180403658862</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="31" t="n">
         <v>0.694536024392415</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="17" t="n">
         <v>8.14967306104231</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="32" t="n">
         <f aca="false">AVERAGE(D5:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="25" t="n">
+      <c r="E10" s="27" t="n">
         <f aca="false">AVERAGE(E5:E9)</f>
         <v>1.41133983495493</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="27" t="n">
         <f aca="false">AVERAGE(F5:F9)</f>
         <v>10.3932156484888</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="28" t="n">
         <f aca="false">AVERAGE(G5:G9)</f>
         <v>0.692881043232584</v>
       </c>
-      <c r="H10" s="27" t="n">
+      <c r="H10" s="29" t="n">
         <f aca="false">AVERAGE(H5:H9)</f>
         <v>8.14765033515906</v>
       </c>
@@ -3950,23 +3957,23 @@
       <c r="C11" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D11" s="31" t="n">
+      <c r="D11" s="33" t="n">
         <f aca="false">STDEV(D5:D9)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">STDEV(E5:E9)</f>
         <v>0.00439921386882577</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <f aca="false">STDEV(F5:F9)</f>
         <v>0.0257457801048861</v>
       </c>
-      <c r="G11" s="32" t="n">
+      <c r="G11" s="34" t="n">
         <f aca="false">STDEV(G5:G9)</f>
         <v>0.00171638534032576</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="13" t="n">
         <f aca="false">STDEV(H5:H9)</f>
         <v>0.00598772016738544</v>
       </c>
@@ -3981,19 +3988,19 @@
       <c r="C13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="22" t="n">
         <v>2057</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E13" s="30" t="n">
         <v>8.17396989080396</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="30" t="n">
         <v>3.99164297815367</v>
       </c>
-      <c r="G13" s="29" t="n">
+      <c r="G13" s="31" t="n">
         <v>0.997910744538417</v>
       </c>
-      <c r="H13" s="16" t="n">
+      <c r="H13" s="17" t="n">
         <v>122.86624734036</v>
       </c>
     </row>
@@ -4007,19 +4014,19 @@
       <c r="C14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="22" t="n">
         <v>2322</v>
       </c>
-      <c r="E14" s="28" t="n">
+      <c r="E14" s="30" t="n">
         <v>8.36617034494946</v>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="30" t="n">
         <v>3.99796981609719</v>
       </c>
-      <c r="G14" s="29" t="n">
+      <c r="G14" s="31" t="n">
         <v>0.999492454024297</v>
       </c>
-      <c r="H14" s="16" t="n">
+      <c r="H14" s="17" t="n">
         <v>125.556280759266</v>
       </c>
     </row>
@@ -4033,19 +4040,19 @@
       <c r="C15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="22" t="n">
         <v>2281</v>
       </c>
-      <c r="E15" s="28" t="n">
+      <c r="E15" s="30" t="n">
         <v>8.43227902433431</v>
       </c>
-      <c r="F15" s="28" t="n">
+      <c r="F15" s="30" t="n">
         <v>3.99856012486839</v>
       </c>
-      <c r="G15" s="29" t="n">
+      <c r="G15" s="31" t="n">
         <v>0.999640031217098</v>
       </c>
-      <c r="H15" s="16" t="n">
+      <c r="H15" s="17" t="n">
         <v>126.529732118686</v>
       </c>
     </row>
@@ -4059,19 +4066,19 @@
       <c r="C16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="22" t="n">
         <v>2405</v>
       </c>
-      <c r="E16" s="28" t="n">
+      <c r="E16" s="30" t="n">
         <v>8.47594504973996</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="30" t="n">
         <v>3.99656930819725</v>
       </c>
-      <c r="G16" s="29" t="n">
+      <c r="G16" s="31" t="n">
         <v>0.999142327049313</v>
       </c>
-      <c r="H16" s="16" t="n">
+      <c r="H16" s="17" t="n">
         <v>127.248313182336</v>
       </c>
     </row>
@@ -4085,49 +4092,49 @@
       <c r="C17" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="22" t="n">
         <v>2182</v>
       </c>
-      <c r="E17" s="28" t="n">
+      <c r="E17" s="30" t="n">
         <v>8.24549095686411</v>
       </c>
-      <c r="F17" s="28" t="n">
+      <c r="F17" s="30" t="n">
         <v>3.98926368262925</v>
       </c>
-      <c r="G17" s="29" t="n">
+      <c r="G17" s="31" t="n">
         <v>0.997315920657312</v>
       </c>
-      <c r="H17" s="16" t="n">
+      <c r="H17" s="17" t="n">
         <v>124.015231072863</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="30" t="n">
+      <c r="D18" s="32" t="n">
         <f aca="false">AVERAGE(D13:D17)</f>
         <v>2249.4</v>
       </c>
-      <c r="E18" s="25" t="n">
+      <c r="E18" s="27" t="n">
         <f aca="false">AVERAGE(E13:E17)</f>
         <v>8.33877105333836</v>
       </c>
-      <c r="F18" s="25" t="n">
+      <c r="F18" s="27" t="n">
         <f aca="false">AVERAGE(F13:F17)</f>
         <v>3.99480118198915</v>
       </c>
-      <c r="G18" s="26" t="n">
+      <c r="G18" s="28" t="n">
         <f aca="false">AVERAGE(G13:G17)</f>
         <v>0.998700295497287</v>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="29" t="n">
         <f aca="false">AVERAGE(H13:H17)</f>
         <v>125.243160894702</v>
       </c>
@@ -4142,23 +4149,23 @@
       <c r="C19" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D19" s="31" t="n">
+      <c r="D19" s="33" t="n">
         <f aca="false">STDEV(D13:D17)</f>
         <v>134.202458993865</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">STDEV(E13:E17)</f>
         <v>0.126660734523659</v>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="F19" s="14" t="n">
         <f aca="false">STDEV(F13:F17)</f>
         <v>0.00412111376314653</v>
       </c>
-      <c r="G19" s="32" t="n">
+      <c r="G19" s="34" t="n">
         <f aca="false">STDEV(G13:G17)</f>
         <v>0.00103027844078667</v>
       </c>
-      <c r="H19" s="12" t="n">
+      <c r="H19" s="13" t="n">
         <f aca="false">STDEV(H13:H17)</f>
         <v>1.79801800274308</v>
       </c>
@@ -4173,19 +4180,19 @@
       <c r="C21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="20" t="n">
+      <c r="D21" s="22" t="n">
         <v>79</v>
       </c>
-      <c r="E21" s="28" t="n">
+      <c r="E21" s="30" t="n">
         <v>1.92326099427399</v>
       </c>
-      <c r="F21" s="28" t="n">
+      <c r="F21" s="30" t="n">
         <v>1.11835315374716</v>
       </c>
-      <c r="G21" s="29" t="n">
+      <c r="G21" s="31" t="n">
         <v>0.838764865310369</v>
       </c>
-      <c r="H21" s="16" t="n">
+      <c r="H21" s="17" t="n">
         <v>103.183559924514</v>
       </c>
     </row>
@@ -4199,19 +4206,19 @@
       <c r="C22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D22" s="20" t="n">
+      <c r="D22" s="22" t="n">
         <v>132</v>
       </c>
-      <c r="E22" s="28" t="n">
+      <c r="E22" s="30" t="n">
         <v>2.19496828076005</v>
       </c>
-      <c r="F22" s="28" t="n">
+      <c r="F22" s="30" t="n">
         <v>1.16998792335286</v>
       </c>
-      <c r="G22" s="29" t="n">
+      <c r="G22" s="31" t="n">
         <v>0.877490942514644</v>
       </c>
-      <c r="H22" s="16" t="n">
+      <c r="H22" s="17" t="n">
         <v>112.563637809349</v>
       </c>
     </row>
@@ -4225,19 +4232,19 @@
       <c r="C23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="22" t="n">
         <v>103</v>
       </c>
-      <c r="E23" s="28" t="n">
+      <c r="E23" s="30" t="n">
         <v>2.16919098238202</v>
       </c>
-      <c r="F23" s="28" t="n">
+      <c r="F23" s="30" t="n">
         <v>1.15695083320826</v>
       </c>
-      <c r="G23" s="29" t="n">
+      <c r="G23" s="31" t="n">
         <v>0.867713124906193</v>
       </c>
-      <c r="H23" s="16" t="n">
+      <c r="H23" s="17" t="n">
         <v>112.495237660193</v>
       </c>
     </row>
@@ -4251,19 +4258,19 @@
       <c r="C24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D24" s="20" t="n">
+      <c r="D24" s="22" t="n">
         <v>163</v>
       </c>
-      <c r="E24" s="28" t="n">
+      <c r="E24" s="30" t="n">
         <v>2.18299558493472</v>
       </c>
-      <c r="F24" s="28" t="n">
+      <c r="F24" s="30" t="n">
         <v>1.15878854510669</v>
       </c>
-      <c r="G24" s="29" t="n">
+      <c r="G24" s="31" t="n">
         <v>0.869091408830016</v>
       </c>
-      <c r="H24" s="16" t="n">
+      <c r="H24" s="17" t="n">
         <v>113.031610166654</v>
       </c>
     </row>
@@ -4277,49 +4284,49 @@
       <c r="C25" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D25" s="22" t="n">
         <v>146</v>
       </c>
-      <c r="E25" s="28" t="n">
+      <c r="E25" s="30" t="n">
         <v>2.18999027237302</v>
       </c>
-      <c r="F25" s="28" t="n">
+      <c r="F25" s="30" t="n">
         <v>1.16263319725305</v>
       </c>
-      <c r="G25" s="29" t="n">
+      <c r="G25" s="31" t="n">
         <v>0.871974897939787</v>
       </c>
-      <c r="H25" s="16" t="n">
+      <c r="H25" s="17" t="n">
         <v>113.018806492743</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D26" s="30" t="n">
+      <c r="D26" s="32" t="n">
         <f aca="false">AVERAGE(D21:D25)</f>
         <v>124.6</v>
       </c>
-      <c r="E26" s="25" t="n">
+      <c r="E26" s="27" t="n">
         <f aca="false">AVERAGE(E21:E25)</f>
         <v>2.13208122294476</v>
       </c>
-      <c r="F26" s="25" t="n">
+      <c r="F26" s="27" t="n">
         <f aca="false">AVERAGE(F21:F25)</f>
         <v>1.1533427305336</v>
       </c>
-      <c r="G26" s="26" t="n">
+      <c r="G26" s="28" t="n">
         <f aca="false">AVERAGE(G21:G25)</f>
         <v>0.865007047900202</v>
       </c>
-      <c r="H26" s="27" t="n">
+      <c r="H26" s="29" t="n">
         <f aca="false">AVERAGE(H21:H25)</f>
         <v>110.85857041069</v>
       </c>
@@ -4334,23 +4341,23 @@
       <c r="C27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="31" t="n">
+      <c r="D27" s="33" t="n">
         <f aca="false">STDEV(D21:D25)</f>
         <v>33.6645213837951</v>
       </c>
-      <c r="E27" s="13" t="n">
+      <c r="E27" s="14" t="n">
         <f aca="false">STDEV(E21:E25)</f>
         <v>0.11713617550825</v>
       </c>
-      <c r="F27" s="13" t="n">
+      <c r="F27" s="14" t="n">
         <f aca="false">STDEV(F21:F25)</f>
         <v>0.0201886168472803</v>
       </c>
-      <c r="G27" s="32" t="n">
+      <c r="G27" s="34" t="n">
         <f aca="false">STDEV(G21:G25)</f>
         <v>0.0151414626354602</v>
       </c>
-      <c r="H27" s="12" t="n">
+      <c r="H27" s="13" t="n">
         <f aca="false">STDEV(H21:H25)</f>
         <v>4.29768665079471</v>
       </c>
@@ -4365,19 +4372,19 @@
       <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="20" t="n">
+      <c r="D29" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="28" t="n">
+      <c r="E29" s="30" t="n">
         <v>1.39488508907472</v>
       </c>
-      <c r="F29" s="28" t="n">
+      <c r="F29" s="30" t="n">
         <v>10.3139826700539</v>
       </c>
-      <c r="G29" s="29" t="n">
+      <c r="G29" s="31" t="n">
         <v>0.687598844670258</v>
       </c>
-      <c r="H29" s="16" t="n">
+      <c r="H29" s="17" t="n">
         <v>8.11452840496641</v>
       </c>
     </row>
@@ -4391,19 +4398,19 @@
       <c r="C30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D30" s="20" t="n">
+      <c r="D30" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="28" t="n">
+      <c r="E30" s="30" t="n">
         <v>1.40656119390452</v>
       </c>
-      <c r="F30" s="28" t="n">
+      <c r="F30" s="30" t="n">
         <v>10.3630483811675</v>
       </c>
-      <c r="G30" s="29" t="n">
+      <c r="G30" s="31" t="n">
         <v>0.690869892077835</v>
       </c>
-      <c r="H30" s="16" t="n">
+      <c r="H30" s="17" t="n">
         <v>8.14371105201414</v>
       </c>
     </row>
@@ -4417,19 +4424,19 @@
       <c r="C31" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="20" t="n">
+      <c r="D31" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="28" t="n">
+      <c r="E31" s="30" t="n">
         <v>1.39854042505951</v>
       </c>
-      <c r="F31" s="28" t="n">
+      <c r="F31" s="30" t="n">
         <v>10.3285490305602</v>
       </c>
-      <c r="G31" s="29" t="n">
+      <c r="G31" s="31" t="n">
         <v>0.68856993537068</v>
       </c>
-      <c r="H31" s="16" t="n">
+      <c r="H31" s="17" t="n">
         <v>8.12431884239402</v>
       </c>
     </row>
@@ -4443,19 +4450,19 @@
       <c r="C32" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D32" s="20" t="n">
+      <c r="D32" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="28" t="n">
+      <c r="E32" s="30" t="n">
         <v>1.40824699461638</v>
       </c>
-      <c r="F32" s="28" t="n">
+      <c r="F32" s="30" t="n">
         <v>10.3729702387231</v>
       </c>
-      <c r="G32" s="29" t="n">
+      <c r="G32" s="31" t="n">
         <v>0.691531349248205</v>
       </c>
-      <c r="H32" s="16" t="n">
+      <c r="H32" s="17" t="n">
         <v>8.14567262147897</v>
       </c>
     </row>
@@ -4469,49 +4476,49 @@
       <c r="C33" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D33" s="20" t="n">
+      <c r="D33" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="28" t="n">
+      <c r="E33" s="30" t="n">
         <v>1.39539099827095</v>
       </c>
-      <c r="F33" s="28" t="n">
+      <c r="F33" s="30" t="n">
         <v>10.3085680685575</v>
       </c>
-      <c r="G33" s="29" t="n">
+      <c r="G33" s="31" t="n">
         <v>0.687237871237167</v>
       </c>
-      <c r="H33" s="16" t="n">
+      <c r="H33" s="17" t="n">
         <v>8.12173517596729</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="14" t="s">
+      <c r="C34" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D34" s="30" t="n">
+      <c r="D34" s="32" t="n">
         <f aca="false">AVERAGE(D29:D33)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="25" t="n">
+      <c r="E34" s="27" t="n">
         <f aca="false">AVERAGE(E29:E33)</f>
         <v>1.40072494018522</v>
       </c>
-      <c r="F34" s="25" t="n">
+      <c r="F34" s="27" t="n">
         <f aca="false">AVERAGE(F29:F33)</f>
         <v>10.3374236778124</v>
       </c>
-      <c r="G34" s="26" t="n">
+      <c r="G34" s="28" t="n">
         <f aca="false">AVERAGE(G29:G33)</f>
         <v>0.689161578520829</v>
       </c>
-      <c r="H34" s="27" t="n">
+      <c r="H34" s="29" t="n">
         <f aca="false">AVERAGE(H29:H33)</f>
         <v>8.12999321936416</v>
       </c>
@@ -4526,23 +4533,23 @@
       <c r="C35" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="31" t="n">
+      <c r="D35" s="33" t="n">
         <f aca="false">STDEV(D29:D33)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="13" t="n">
+      <c r="E35" s="14" t="n">
         <f aca="false">STDEV(E29:E33)</f>
         <v>0.00628430712197881</v>
       </c>
-      <c r="F35" s="13" t="n">
+      <c r="F35" s="14" t="n">
         <f aca="false">STDEV(F29:F33)</f>
         <v>0.0290734836606808</v>
       </c>
-      <c r="G35" s="32" t="n">
+      <c r="G35" s="34" t="n">
         <f aca="false">STDEV(G29:G33)</f>
         <v>0.00193823224404539</v>
       </c>
-      <c r="H35" s="12" t="n">
+      <c r="H35" s="13" t="n">
         <f aca="false">STDEV(H29:H33)</f>
         <v>0.0139066252411523</v>
       </c>
@@ -4557,19 +4564,19 @@
       <c r="C37" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="20" t="n">
+      <c r="D37" s="22" t="n">
         <v>19</v>
       </c>
-      <c r="E37" s="28" t="n">
+      <c r="E37" s="30" t="n">
         <v>2.60866603726795</v>
       </c>
-      <c r="F37" s="28" t="n">
+      <c r="F37" s="30" t="n">
         <v>3.19126005156441</v>
       </c>
-      <c r="G37" s="29" t="n">
+      <c r="G37" s="31" t="n">
         <v>0.797815012891104</v>
       </c>
-      <c r="H37" s="16" t="n">
+      <c r="H37" s="17" t="n">
         <v>49.0464455127523</v>
       </c>
     </row>
@@ -4583,19 +4590,19 @@
       <c r="C38" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="20" t="n">
+      <c r="D38" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="E38" s="28" t="n">
+      <c r="E38" s="30" t="n">
         <v>2.82534499097601</v>
       </c>
-      <c r="F38" s="28" t="n">
+      <c r="F38" s="30" t="n">
         <v>3.30026829017066</v>
       </c>
-      <c r="G38" s="29" t="n">
+      <c r="G38" s="31" t="n">
         <v>0.825067072542664</v>
       </c>
-      <c r="H38" s="16" t="n">
+      <c r="H38" s="17" t="n">
         <v>51.3657328900963</v>
       </c>
     </row>
@@ -4609,19 +4616,19 @@
       <c r="C39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D39" s="20" t="n">
+      <c r="D39" s="22" t="n">
         <v>33</v>
       </c>
-      <c r="E39" s="28" t="n">
+      <c r="E39" s="30" t="n">
         <v>2.85359245810866</v>
       </c>
-      <c r="F39" s="28" t="n">
+      <c r="F39" s="30" t="n">
         <v>3.28467263694278</v>
       </c>
-      <c r="G39" s="29" t="n">
+      <c r="G39" s="31" t="n">
         <v>0.821168159235695</v>
       </c>
-      <c r="H39" s="16" t="n">
+      <c r="H39" s="17" t="n">
         <v>52.1256047134971</v>
       </c>
     </row>
@@ -4635,19 +4642,19 @@
       <c r="C40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D40" s="20" t="n">
+      <c r="D40" s="22" t="n">
         <v>43</v>
       </c>
-      <c r="E40" s="28" t="n">
+      <c r="E40" s="30" t="n">
         <v>3.09387009388168</v>
       </c>
-      <c r="F40" s="28" t="n">
+      <c r="F40" s="30" t="n">
         <v>3.33964538777848</v>
       </c>
-      <c r="G40" s="29" t="n">
+      <c r="G40" s="31" t="n">
         <v>0.834911346944621</v>
       </c>
-      <c r="H40" s="16" t="n">
+      <c r="H40" s="17" t="n">
         <v>55.5844061504932</v>
       </c>
     </row>
@@ -4661,49 +4668,49 @@
       <c r="C41" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D41" s="20" t="n">
+      <c r="D41" s="22" t="n">
         <v>30</v>
       </c>
-      <c r="E41" s="28" t="n">
+      <c r="E41" s="30" t="n">
         <v>2.82902707642674</v>
       </c>
-      <c r="F41" s="28" t="n">
+      <c r="F41" s="30" t="n">
         <v>3.29777554828438</v>
       </c>
-      <c r="G41" s="29" t="n">
+      <c r="G41" s="31" t="n">
         <v>0.824443887071095</v>
       </c>
-      <c r="H41" s="16" t="n">
+      <c r="H41" s="17" t="n">
         <v>51.4715516869879</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="14" t="s">
+      <c r="A42" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="C42" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D42" s="30" t="n">
+      <c r="D42" s="32" t="n">
         <f aca="false">AVERAGE(D37:D41)</f>
         <v>30</v>
       </c>
-      <c r="E42" s="25" t="n">
+      <c r="E42" s="27" t="n">
         <f aca="false">AVERAGE(E37:E41)</f>
         <v>2.84210013133221</v>
       </c>
-      <c r="F42" s="25" t="n">
+      <c r="F42" s="27" t="n">
         <f aca="false">AVERAGE(F37:F41)</f>
         <v>3.28272438294814</v>
       </c>
-      <c r="G42" s="26" t="n">
+      <c r="G42" s="28" t="n">
         <f aca="false">AVERAGE(G37:G41)</f>
         <v>0.820681095737036</v>
       </c>
-      <c r="H42" s="27" t="n">
+      <c r="H42" s="29" t="n">
         <f aca="false">AVERAGE(H37:H41)</f>
         <v>51.9187481907654</v>
       </c>
@@ -4718,23 +4725,23 @@
       <c r="C43" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D43" s="31" t="n">
+      <c r="D43" s="33" t="n">
         <f aca="false">STDEV(D37:D41)</f>
         <v>9</v>
       </c>
-      <c r="E43" s="13" t="n">
+      <c r="E43" s="14" t="n">
         <f aca="false">STDEV(E37:E41)</f>
         <v>0.172092492123722</v>
       </c>
-      <c r="F43" s="13" t="n">
+      <c r="F43" s="14" t="n">
         <f aca="false">STDEV(F37:F41)</f>
         <v>0.0550995613834784</v>
       </c>
-      <c r="G43" s="32" t="n">
+      <c r="G43" s="34" t="n">
         <f aca="false">STDEV(G37:G41)</f>
         <v>0.0137748903458695</v>
       </c>
-      <c r="H43" s="12" t="n">
+      <c r="H43" s="13" t="n">
         <f aca="false">STDEV(H37:H41)</f>
         <v>2.3577410379746</v>
       </c>
@@ -4749,19 +4756,19 @@
       <c r="C45" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="20" t="n">
+      <c r="D45" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="E45" s="28" t="n">
+      <c r="E45" s="30" t="n">
         <v>1.30476270994767</v>
       </c>
-      <c r="F45" s="28" t="n">
+      <c r="F45" s="30" t="n">
         <v>0.957204790250873</v>
       </c>
-      <c r="G45" s="29" t="n">
+      <c r="G45" s="31" t="n">
         <v>0.717903592688155</v>
       </c>
-      <c r="H45" s="16" t="n">
+      <c r="H45" s="17" t="n">
         <v>81.7858031992739</v>
       </c>
     </row>
@@ -4775,19 +4782,19 @@
       <c r="C46" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D46" s="20" t="n">
+      <c r="D46" s="22" t="n">
         <v>32</v>
       </c>
-      <c r="E46" s="28" t="n">
+      <c r="E46" s="30" t="n">
         <v>1.3751723417863</v>
       </c>
-      <c r="F46" s="28" t="n">
+      <c r="F46" s="30" t="n">
         <v>0.975368869097814</v>
       </c>
-      <c r="G46" s="29" t="n">
+      <c r="G46" s="31" t="n">
         <v>0.731526651823361</v>
       </c>
-      <c r="H46" s="16" t="n">
+      <c r="H46" s="17" t="n">
         <v>84.5939860511415</v>
       </c>
     </row>
@@ -4801,19 +4808,19 @@
       <c r="C47" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D47" s="20" t="n">
+      <c r="D47" s="22" t="n">
         <v>33</v>
       </c>
-      <c r="E47" s="28" t="n">
+      <c r="E47" s="30" t="n">
         <v>1.39335862489791</v>
       </c>
-      <c r="F47" s="28" t="n">
+      <c r="F47" s="30" t="n">
         <v>0.970303494294256</v>
       </c>
-      <c r="G47" s="29" t="n">
+      <c r="G47" s="31" t="n">
         <v>0.727727620720692</v>
       </c>
-      <c r="H47" s="16" t="n">
+      <c r="H47" s="17" t="n">
         <v>86.1601735802068</v>
       </c>
     </row>
@@ -4827,19 +4834,19 @@
       <c r="C48" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D48" s="20" t="n">
+      <c r="D48" s="22" t="n">
         <v>35</v>
       </c>
-      <c r="E48" s="28" t="n">
+      <c r="E48" s="30" t="n">
         <v>1.38930425101755</v>
       </c>
-      <c r="F48" s="28" t="n">
+      <c r="F48" s="30" t="n">
         <v>0.972201327156678</v>
       </c>
-      <c r="G48" s="29" t="n">
+      <c r="G48" s="31" t="n">
         <v>0.729150995367509</v>
       </c>
-      <c r="H48" s="16" t="n">
+      <c r="H48" s="17" t="n">
         <v>85.7417622591037</v>
       </c>
     </row>
@@ -4853,49 +4860,49 @@
       <c r="C49" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D49" s="20" t="n">
+      <c r="D49" s="22" t="n">
         <v>28</v>
       </c>
-      <c r="E49" s="28" t="n">
+      <c r="E49" s="30" t="n">
         <v>1.48083520571888</v>
       </c>
-      <c r="F49" s="28" t="n">
+      <c r="F49" s="30" t="n">
         <v>0.995720294714835</v>
       </c>
-      <c r="G49" s="29" t="n">
+      <c r="G49" s="31" t="n">
         <v>0.746790221036126</v>
       </c>
-      <c r="H49" s="16" t="n">
+      <c r="H49" s="17" t="n">
         <v>89.2319990008625</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="14" t="s">
+      <c r="A50" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B50" s="14" t="s">
+      <c r="B50" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="14" t="s">
+      <c r="C50" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D50" s="30" t="n">
+      <c r="D50" s="32" t="n">
         <f aca="false">AVERAGE(D45:D49)</f>
         <v>28.6</v>
       </c>
-      <c r="E50" s="25" t="n">
+      <c r="E50" s="27" t="n">
         <f aca="false">AVERAGE(E45:E49)</f>
         <v>1.38868662667366</v>
       </c>
-      <c r="F50" s="25" t="n">
+      <c r="F50" s="27" t="n">
         <f aca="false">AVERAGE(F45:F49)</f>
         <v>0.974159755102891</v>
       </c>
-      <c r="G50" s="26" t="n">
+      <c r="G50" s="28" t="n">
         <f aca="false">AVERAGE(G45:G49)</f>
         <v>0.730619816327168</v>
       </c>
-      <c r="H50" s="27" t="n">
+      <c r="H50" s="29" t="n">
         <f aca="false">AVERAGE(H45:H49)</f>
         <v>85.5027448181177</v>
       </c>
@@ -4910,23 +4917,23 @@
       <c r="C51" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D51" s="31" t="n">
+      <c r="D51" s="33" t="n">
         <f aca="false">STDEV(D45:D49)</f>
         <v>8.01872807869178</v>
       </c>
-      <c r="E51" s="13" t="n">
+      <c r="E51" s="14" t="n">
         <f aca="false">STDEV(E45:E49)</f>
         <v>0.0627284412008175</v>
       </c>
-      <c r="F51" s="13" t="n">
+      <c r="F51" s="14" t="n">
         <f aca="false">STDEV(F45:F49)</f>
         <v>0.0138969047416033</v>
       </c>
-      <c r="G51" s="32" t="n">
+      <c r="G51" s="34" t="n">
         <f aca="false">STDEV(G45:G49)</f>
         <v>0.0104226785562025</v>
       </c>
-      <c r="H51" s="12" t="n">
+      <c r="H51" s="13" t="n">
         <f aca="false">STDEV(H45:H49)</f>
         <v>2.69435410480351</v>
       </c>
@@ -4934,7 +4941,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>